<commit_message>
update: 2026/06/07 周日 14:17:56.87
</commit_message>
<xml_diff>
--- a/source/8、绩效异常岗位/1、装车岗/装车岗-6月.xlsx
+++ b/source/8、绩效异常岗位/1、装车岗/装车岗-6月.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="75">
   <si>
     <t>数据日期</t>
   </si>
@@ -64,18 +64,12 @@
     <t>银川</t>
   </si>
   <si>
-    <t>119.2</t>
-  </si>
-  <si>
     <t>辽宁区</t>
   </si>
   <si>
     <t>盘锦</t>
   </si>
   <si>
-    <t>90.1</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -85,208 +79,181 @@
     <t>太原</t>
   </si>
   <si>
-    <t>143.9</t>
-  </si>
-  <si>
     <t>河北区</t>
   </si>
   <si>
     <t>邢邯</t>
   </si>
   <si>
-    <t>133</t>
-  </si>
-  <si>
     <t>石家庄</t>
   </si>
   <si>
-    <t>154.1</t>
-  </si>
-  <si>
     <t>湖南区</t>
   </si>
   <si>
     <t>衡阳</t>
   </si>
   <si>
-    <t>114.8</t>
-  </si>
-  <si>
     <t>黑龙江区</t>
   </si>
   <si>
     <t>哈尔滨</t>
   </si>
   <si>
-    <t>132.7</t>
-  </si>
-  <si>
     <t>天津区</t>
   </si>
   <si>
     <t>天津</t>
   </si>
   <si>
-    <t>114.9</t>
-  </si>
-  <si>
     <t>常德</t>
   </si>
   <si>
-    <t>107.6</t>
-  </si>
-  <si>
     <t>河南区</t>
   </si>
   <si>
     <t>商丘</t>
   </si>
   <si>
-    <t>130.7</t>
-  </si>
-  <si>
     <t>贵州区</t>
   </si>
   <si>
     <t>贵阳</t>
   </si>
   <si>
-    <t>212.6</t>
-  </si>
-  <si>
     <t>安徽区</t>
   </si>
   <si>
     <t>安庆</t>
   </si>
   <si>
-    <t>103.9</t>
-  </si>
-  <si>
     <t>陕西区</t>
   </si>
   <si>
     <t>西安</t>
   </si>
   <si>
-    <t>122.5</t>
-  </si>
-  <si>
     <t>肃宁</t>
   </si>
   <si>
-    <t>113.6</t>
-  </si>
-  <si>
     <t>湖北区</t>
   </si>
   <si>
     <t>武汉</t>
   </si>
   <si>
-    <t>144.8</t>
-  </si>
-  <si>
     <t>武昌</t>
   </si>
   <si>
-    <t>113.9</t>
-  </si>
-  <si>
     <t>广西区</t>
   </si>
   <si>
     <t>柳州</t>
   </si>
   <si>
-    <t>82.7</t>
-  </si>
-  <si>
     <t>江苏区</t>
   </si>
   <si>
     <t>淮安</t>
   </si>
   <si>
-    <t>187.3</t>
-  </si>
-  <si>
     <t>重庆区</t>
   </si>
   <si>
     <t>重庆</t>
   </si>
   <si>
-    <t>169.6</t>
-  </si>
-  <si>
     <t>浙北区</t>
   </si>
   <si>
     <t>东方天地港</t>
   </si>
   <si>
-    <t>166</t>
-  </si>
-  <si>
     <t>四川区</t>
   </si>
   <si>
     <t>成都</t>
   </si>
   <si>
-    <t>210.8</t>
-  </si>
-  <si>
     <t>南通</t>
   </si>
   <si>
-    <t>169.8</t>
-  </si>
-  <si>
     <t>浙南区</t>
   </si>
   <si>
     <t>临海</t>
   </si>
   <si>
-    <t>172.7</t>
-  </si>
-  <si>
     <t>义乌</t>
   </si>
   <si>
-    <t>220.2</t>
-  </si>
-  <si>
     <t>粤东区</t>
   </si>
   <si>
     <t>揭阳</t>
   </si>
   <si>
-    <t>216.2</t>
-  </si>
-  <si>
     <t>广东区</t>
   </si>
   <si>
     <t>广州</t>
   </si>
   <si>
-    <t>226.1</t>
-  </si>
-  <si>
     <t>合肥</t>
   </si>
   <si>
-    <t>182.4</t>
-  </si>
-  <si>
     <t>南京</t>
   </si>
   <si>
-    <t>200</t>
+    <t>2026-06-02</t>
+  </si>
+  <si>
+    <t>江西区</t>
+  </si>
+  <si>
+    <t>赣州</t>
+  </si>
+  <si>
+    <t>芜湖</t>
+  </si>
+  <si>
+    <t>2026-06-03</t>
+  </si>
+  <si>
+    <t>山东区</t>
+  </si>
+  <si>
+    <t>潍坊</t>
+  </si>
+  <si>
+    <t>深圳</t>
+  </si>
+  <si>
+    <t>临沂</t>
+  </si>
+  <si>
+    <t>2026-06-04</t>
+  </si>
+  <si>
+    <t>甘肃区</t>
+  </si>
+  <si>
+    <t>兰州</t>
+  </si>
+  <si>
+    <t>长治</t>
+  </si>
+  <si>
+    <t>宁波</t>
+  </si>
+  <si>
+    <t>上海区</t>
+  </si>
+  <si>
+    <t>浦东</t>
+  </si>
+  <si>
+    <t>2026-06-05</t>
   </si>
 </sst>
 </file>
@@ -1220,7 +1187,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr defaultColWidth="12.6363636363636" defaultRowHeight="20" customHeight="1" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="16384" width="12.6363636363636" style="1" customWidth="1"/>
@@ -1262,8 +1229,8 @@
       <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>11</v>
+      <c r="D2" s="1">
+        <v>119.2</v>
       </c>
       <c r="E2" s="1">
         <v>285</v>
@@ -1283,13 +1250,13 @@
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>14</v>
+      <c r="D3" s="1">
+        <v>90.1</v>
       </c>
       <c r="E3" s="1">
         <v>117.7</v>
@@ -1298,10 +1265,10 @@
         <v>30.5</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" customHeight="1" spans="1:8">
@@ -1309,13 +1276,13 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="D4" s="1">
+        <v>143.9</v>
       </c>
       <c r="E4" s="1">
         <v>183.4</v>
@@ -1335,13 +1302,13 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
+      </c>
+      <c r="D5" s="1">
+        <v>133</v>
       </c>
       <c r="E5" s="1">
         <v>166.6</v>
@@ -1361,13 +1328,13 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="D6" s="1">
+        <v>154.1</v>
       </c>
       <c r="E6" s="1">
         <v>187.9</v>
@@ -1387,13 +1354,13 @@
         <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
+      </c>
+      <c r="D7" s="1">
+        <v>114.8</v>
       </c>
       <c r="E7" s="1">
         <v>139.7</v>
@@ -1402,10 +1369,10 @@
         <v>21.7</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="1:8">
@@ -1413,13 +1380,13 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
+      </c>
+      <c r="D8" s="1">
+        <v>132.7</v>
       </c>
       <c r="E8" s="1">
         <v>160.2</v>
@@ -1439,13 +1406,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
+      </c>
+      <c r="D9" s="1">
+        <v>114.9</v>
       </c>
       <c r="E9" s="1">
         <v>138.1</v>
@@ -1454,10 +1421,10 @@
         <v>20.2</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="1:8">
@@ -1465,13 +1432,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>34</v>
+        <v>25</v>
+      </c>
+      <c r="D10" s="1">
+        <v>107.6</v>
       </c>
       <c r="E10" s="1">
         <v>129.2</v>
@@ -1480,10 +1447,10 @@
         <v>20</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" customHeight="1" spans="1:8">
@@ -1491,13 +1458,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>37</v>
+        <v>27</v>
+      </c>
+      <c r="D11" s="1">
+        <v>130.7</v>
       </c>
       <c r="E11" s="1">
         <v>153.1</v>
@@ -1506,10 +1473,10 @@
         <v>17.1</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="1:8">
@@ -1517,13 +1484,13 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
+      </c>
+      <c r="D12" s="1">
+        <v>212.6</v>
       </c>
       <c r="E12" s="1">
         <v>244.7</v>
@@ -1543,13 +1510,13 @@
         <v>8</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>43</v>
+        <v>31</v>
+      </c>
+      <c r="D13" s="1">
+        <v>103.9</v>
       </c>
       <c r="E13" s="1">
         <v>119.6</v>
@@ -1558,10 +1525,10 @@
         <v>15</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="1:8">
@@ -1569,13 +1536,13 @@
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>46</v>
+        <v>33</v>
+      </c>
+      <c r="D14" s="1">
+        <v>122.5</v>
       </c>
       <c r="E14" s="1">
         <v>140.6</v>
@@ -1584,10 +1551,10 @@
         <v>14.8</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" customHeight="1" spans="1:8">
@@ -1595,13 +1562,13 @@
         <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
+      </c>
+      <c r="D15" s="1">
+        <v>113.6</v>
       </c>
       <c r="E15" s="1">
         <v>128.8</v>
@@ -1610,10 +1577,10 @@
         <v>13.3</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" customHeight="1" spans="1:8">
@@ -1621,13 +1588,13 @@
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
+      </c>
+      <c r="D16" s="1">
+        <v>144.8</v>
       </c>
       <c r="E16" s="1">
         <v>163.2</v>
@@ -1647,13 +1614,13 @@
         <v>8</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
+      </c>
+      <c r="D17" s="1">
+        <v>113.9</v>
       </c>
       <c r="E17" s="1">
         <v>126.9</v>
@@ -1662,10 +1629,10 @@
         <v>11.4</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="1:8">
@@ -1673,13 +1640,13 @@
         <v>8</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>56</v>
+        <v>39</v>
+      </c>
+      <c r="D18" s="1">
+        <v>82.7</v>
       </c>
       <c r="E18" s="1">
         <v>92.1</v>
@@ -1688,10 +1655,10 @@
         <v>11.3</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" customHeight="1" spans="1:8">
@@ -1699,13 +1666,13 @@
         <v>8</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>59</v>
+        <v>41</v>
+      </c>
+      <c r="D19" s="1">
+        <v>187.3</v>
       </c>
       <c r="E19" s="1">
         <v>205.3</v>
@@ -1725,13 +1692,13 @@
         <v>8</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>62</v>
+        <v>43</v>
+      </c>
+      <c r="D20" s="1">
+        <v>169.6</v>
       </c>
       <c r="E20" s="1">
         <v>179.8</v>
@@ -1751,13 +1718,13 @@
         <v>8</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>65</v>
+        <v>45</v>
+      </c>
+      <c r="D21" s="1">
+        <v>166</v>
       </c>
       <c r="E21" s="1">
         <v>176</v>
@@ -1777,13 +1744,13 @@
         <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>68</v>
+        <v>47</v>
+      </c>
+      <c r="D22" s="1">
+        <v>210.8</v>
       </c>
       <c r="E22" s="1">
         <v>219.7</v>
@@ -1803,13 +1770,13 @@
         <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>70</v>
+        <v>48</v>
+      </c>
+      <c r="D23" s="1">
+        <v>169.8</v>
       </c>
       <c r="E23" s="1">
         <v>176.6</v>
@@ -1829,13 +1796,13 @@
         <v>8</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>73</v>
+        <v>50</v>
+      </c>
+      <c r="D24" s="1">
+        <v>172.7</v>
       </c>
       <c r="E24" s="1">
         <v>174.3</v>
@@ -1855,13 +1822,13 @@
         <v>8</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>75</v>
+        <v>51</v>
+      </c>
+      <c r="D25" s="1">
+        <v>220.2</v>
       </c>
       <c r="E25" s="1">
         <v>219.2</v>
@@ -1881,13 +1848,13 @@
         <v>8</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>78</v>
+        <v>53</v>
+      </c>
+      <c r="D26" s="1">
+        <v>216.2</v>
       </c>
       <c r="E26" s="1">
         <v>213.2</v>
@@ -1907,13 +1874,13 @@
         <v>8</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>79</v>
+        <v>54</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>81</v>
+        <v>55</v>
+      </c>
+      <c r="D27" s="1">
+        <v>226.1</v>
       </c>
       <c r="E27" s="1">
         <v>221.9</v>
@@ -1933,13 +1900,13 @@
         <v>8</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>83</v>
+        <v>56</v>
+      </c>
+      <c r="D28" s="1">
+        <v>182.4</v>
       </c>
       <c r="E28" s="1">
         <v>178.7</v>
@@ -1959,13 +1926,13 @@
         <v>8</v>
       </c>
       <c r="B29" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>85</v>
+      <c r="D29" s="1">
+        <v>200</v>
       </c>
       <c r="E29" s="1">
         <v>186.4</v>
@@ -1978,6 +1945,2866 @@
       </c>
       <c r="H29" s="1">
         <v>19.1</v>
+      </c>
+    </row>
+    <row r="30" customHeight="1" spans="1:8">
+      <c r="A30" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="1">
+        <v>119.2</v>
+      </c>
+      <c r="E30" s="1">
+        <v>331.1</v>
+      </c>
+      <c r="F30" s="1">
+        <v>177.7</v>
+      </c>
+      <c r="G30" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H30" s="1">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" customHeight="1" spans="1:8">
+      <c r="A31" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="1">
+        <v>133</v>
+      </c>
+      <c r="E31" s="1">
+        <v>164.1</v>
+      </c>
+      <c r="F31" s="1">
+        <v>23.3</v>
+      </c>
+      <c r="G31" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H31" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="32" customHeight="1" spans="1:8">
+      <c r="A32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="1">
+        <v>88.7</v>
+      </c>
+      <c r="E32" s="1">
+        <v>105.1</v>
+      </c>
+      <c r="F32" s="1">
+        <v>18.4</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" customHeight="1" spans="1:8">
+      <c r="A33" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D33" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="E33" s="1">
+        <v>144.7</v>
+      </c>
+      <c r="F33" s="1">
+        <v>18.1</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" customHeight="1" spans="1:8">
+      <c r="A34" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D34" s="1">
+        <v>130.7</v>
+      </c>
+      <c r="E34" s="1">
+        <v>153.8</v>
+      </c>
+      <c r="F34" s="1">
+        <v>17.6</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" customHeight="1" spans="1:8">
+      <c r="A35" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="1">
+        <v>154.1</v>
+      </c>
+      <c r="E35" s="1">
+        <v>179.7</v>
+      </c>
+      <c r="F35" s="1">
+        <v>16.6</v>
+      </c>
+      <c r="G35" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H35" s="1">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="36" customHeight="1" spans="1:8">
+      <c r="A36" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" s="1">
+        <v>136.7</v>
+      </c>
+      <c r="E36" s="1">
+        <v>159.5</v>
+      </c>
+      <c r="F36" s="1">
+        <v>16.6</v>
+      </c>
+      <c r="G36" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H36" s="1">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="37" customHeight="1" spans="1:8">
+      <c r="A37" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D37" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="E37" s="1">
+        <v>243.7</v>
+      </c>
+      <c r="F37" s="1">
+        <v>14.6</v>
+      </c>
+      <c r="G37" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H37" s="1">
+        <v>56.8</v>
+      </c>
+    </row>
+    <row r="38" customHeight="1" spans="1:8">
+      <c r="A38" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38" s="1">
+        <v>107.6</v>
+      </c>
+      <c r="E38" s="1">
+        <v>122.7</v>
+      </c>
+      <c r="F38" s="1">
+        <v>14</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" customHeight="1" spans="1:8">
+      <c r="A39" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D39" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="E39" s="1">
+        <v>208.4</v>
+      </c>
+      <c r="F39" s="1">
+        <v>11.3</v>
+      </c>
+      <c r="G39" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H39" s="1">
+        <v>34.1</v>
+      </c>
+    </row>
+    <row r="40" customHeight="1" spans="1:8">
+      <c r="A40" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="E40" s="1">
+        <v>115.6</v>
+      </c>
+      <c r="F40" s="1">
+        <v>11.2</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" customHeight="1" spans="1:8">
+      <c r="A41" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" s="1">
+        <v>114.8</v>
+      </c>
+      <c r="E41" s="1">
+        <v>127.5</v>
+      </c>
+      <c r="F41" s="1">
+        <v>11</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" customHeight="1" spans="1:8">
+      <c r="A42" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D42" s="1">
+        <v>100.7</v>
+      </c>
+      <c r="E42" s="1">
+        <v>111.8</v>
+      </c>
+      <c r="F42" s="1">
+        <v>11</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" customHeight="1" spans="1:8">
+      <c r="A43" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D43" s="1">
+        <v>113.9</v>
+      </c>
+      <c r="E43" s="1">
+        <v>125.9</v>
+      </c>
+      <c r="F43" s="1">
+        <v>10.5</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" customHeight="1" spans="1:8">
+      <c r="A44" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D44" s="1">
+        <v>166</v>
+      </c>
+      <c r="E44" s="1">
+        <v>179.5</v>
+      </c>
+      <c r="F44" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="G44" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H44" s="1">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="45" customHeight="1" spans="1:8">
+      <c r="A45" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D45" s="1">
+        <v>169.8</v>
+      </c>
+      <c r="E45" s="1">
+        <v>181.8</v>
+      </c>
+      <c r="F45" s="1">
+        <v>7</v>
+      </c>
+      <c r="G45" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H45" s="1">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="46" customHeight="1" spans="1:8">
+      <c r="A46" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D46" s="1">
+        <v>212.3</v>
+      </c>
+      <c r="E46" s="1">
+        <v>226.9</v>
+      </c>
+      <c r="F46" s="1">
+        <v>6.8</v>
+      </c>
+      <c r="G46" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H46" s="1">
+        <v>45.9</v>
+      </c>
+    </row>
+    <row r="47" customHeight="1" spans="1:8">
+      <c r="A47" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D47" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="E47" s="1">
+        <v>231.7</v>
+      </c>
+      <c r="F47" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="G47" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H47" s="1">
+        <v>49.1</v>
+      </c>
+    </row>
+    <row r="48" customHeight="1" spans="1:8">
+      <c r="A48" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D48" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="E48" s="1">
+        <v>177.3</v>
+      </c>
+      <c r="F48" s="1">
+        <v>5</v>
+      </c>
+      <c r="G48" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H48" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" customHeight="1" spans="1:8">
+      <c r="A49" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D49" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="E49" s="1">
+        <v>222.9</v>
+      </c>
+      <c r="F49" s="1">
+        <v>-1.4</v>
+      </c>
+      <c r="G49" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H49" s="1">
+        <v>43.4</v>
+      </c>
+    </row>
+    <row r="50" customHeight="1" spans="1:8">
+      <c r="A50" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D50" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="E50" s="1">
+        <v>212.9</v>
+      </c>
+      <c r="F50" s="1">
+        <v>-1.4</v>
+      </c>
+      <c r="G50" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H50" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="51" customHeight="1" spans="1:8">
+      <c r="A51" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D51" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="E51" s="1">
+        <v>177.5</v>
+      </c>
+      <c r="F51" s="1">
+        <v>-2.6</v>
+      </c>
+      <c r="G51" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H51" s="1">
+        <v>14.2</v>
+      </c>
+    </row>
+    <row r="52" customHeight="1" spans="1:8">
+      <c r="A52" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D52" s="1">
+        <v>200</v>
+      </c>
+      <c r="E52" s="1">
+        <v>192.6</v>
+      </c>
+      <c r="F52" s="1">
+        <v>-3.6</v>
+      </c>
+      <c r="G52" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H52" s="1">
+        <v>23.9</v>
+      </c>
+    </row>
+    <row r="53" customHeight="1" spans="1:8">
+      <c r="A53" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D53" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="E53" s="1">
+        <v>192.2</v>
+      </c>
+      <c r="F53" s="1">
+        <v>-3.8</v>
+      </c>
+      <c r="G53" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H53" s="1">
+        <v>23.6</v>
+      </c>
+    </row>
+    <row r="54" customHeight="1" spans="1:8">
+      <c r="A54" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D54" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="E54" s="1">
+        <v>176.1</v>
+      </c>
+      <c r="F54" s="1">
+        <v>-4.9</v>
+      </c>
+      <c r="G54" s="1">
+        <v>155.4</v>
+      </c>
+      <c r="H54" s="1">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="55" customHeight="1" spans="1:8">
+      <c r="A55" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" s="1">
+        <v>119.2</v>
+      </c>
+      <c r="E55" s="1">
+        <v>327</v>
+      </c>
+      <c r="F55" s="1">
+        <v>174.2</v>
+      </c>
+      <c r="G55" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H55" s="1">
+        <v>109.4</v>
+      </c>
+    </row>
+    <row r="56" customHeight="1" spans="1:8">
+      <c r="A56" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D56" s="1">
+        <v>130.7</v>
+      </c>
+      <c r="E56" s="1">
+        <v>157.7</v>
+      </c>
+      <c r="F56" s="1">
+        <v>20.5</v>
+      </c>
+      <c r="G56" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H56" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" customHeight="1" spans="1:8">
+      <c r="A57" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D57" s="1">
+        <v>133</v>
+      </c>
+      <c r="E57" s="1">
+        <v>159</v>
+      </c>
+      <c r="F57" s="1">
+        <v>19.5</v>
+      </c>
+      <c r="G57" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H57" s="1">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="58" customHeight="1" spans="1:8">
+      <c r="A58" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D58" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="E58" s="1">
+        <v>146.3</v>
+      </c>
+      <c r="F58" s="1">
+        <v>19.4</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" customHeight="1" spans="1:8">
+      <c r="A59" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D59" s="1">
+        <v>88.7</v>
+      </c>
+      <c r="E59" s="1">
+        <v>102.6</v>
+      </c>
+      <c r="F59" s="1">
+        <v>15.6</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" customHeight="1" spans="1:8">
+      <c r="A60" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D60" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="E60" s="1">
+        <v>245.5</v>
+      </c>
+      <c r="F60" s="1">
+        <v>15.4</v>
+      </c>
+      <c r="G60" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H60" s="1">
+        <v>57.3</v>
+      </c>
+    </row>
+    <row r="61" customHeight="1" spans="1:8">
+      <c r="A61" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="1">
+        <v>154.1</v>
+      </c>
+      <c r="E61" s="1">
+        <v>177.2</v>
+      </c>
+      <c r="F61" s="1">
+        <v>14.9</v>
+      </c>
+      <c r="G61" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H61" s="1">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="62" customHeight="1" spans="1:8">
+      <c r="A62" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D62" s="1">
+        <v>100.7</v>
+      </c>
+      <c r="E62" s="1">
+        <v>115.4</v>
+      </c>
+      <c r="F62" s="1">
+        <v>14.6</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" customHeight="1" spans="1:8">
+      <c r="A63" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D63" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="E63" s="1">
+        <v>116.7</v>
+      </c>
+      <c r="F63" s="1">
+        <v>12.2</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="64" customHeight="1" spans="1:8">
+      <c r="A64" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D64" s="1">
+        <v>136.7</v>
+      </c>
+      <c r="E64" s="1">
+        <v>152.7</v>
+      </c>
+      <c r="F64" s="1">
+        <v>11.7</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="65" customHeight="1" spans="1:8">
+      <c r="A65" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D65" s="1">
+        <v>113.9</v>
+      </c>
+      <c r="E65" s="1">
+        <v>126.6</v>
+      </c>
+      <c r="F65" s="1">
+        <v>11.1</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" customHeight="1" spans="1:8">
+      <c r="A66" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D66" s="1">
+        <v>107.6</v>
+      </c>
+      <c r="E66" s="1">
+        <v>119.6</v>
+      </c>
+      <c r="F66" s="1">
+        <v>11</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" customHeight="1" spans="1:8">
+      <c r="A67" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D67" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="E67" s="1">
+        <v>164.7</v>
+      </c>
+      <c r="F67" s="1">
+        <v>10.9</v>
+      </c>
+      <c r="G67" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H67" s="1">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="68" customHeight="1" spans="1:8">
+      <c r="A68" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D68" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="E68" s="1">
+        <v>206.4</v>
+      </c>
+      <c r="F68" s="1">
+        <v>10.2</v>
+      </c>
+      <c r="G68" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H68" s="1">
+        <v>32.2</v>
+      </c>
+    </row>
+    <row r="69" customHeight="1" spans="1:8">
+      <c r="A69" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D69" s="1">
+        <v>149.4</v>
+      </c>
+      <c r="E69" s="1">
+        <v>164.6</v>
+      </c>
+      <c r="F69" s="1">
+        <v>10.1</v>
+      </c>
+      <c r="G69" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H69" s="1">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="70" customHeight="1" spans="1:8">
+      <c r="A70" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70" s="1">
+        <v>169.8</v>
+      </c>
+      <c r="E70" s="1">
+        <v>184.7</v>
+      </c>
+      <c r="F70" s="1">
+        <v>8.7</v>
+      </c>
+      <c r="G70" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H70" s="1">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="71" customHeight="1" spans="1:8">
+      <c r="A71" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D71" s="1">
+        <v>166</v>
+      </c>
+      <c r="E71" s="1">
+        <v>180.2</v>
+      </c>
+      <c r="F71" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="G71" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H71" s="1">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="72" customHeight="1" spans="1:8">
+      <c r="A72" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D72" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="E72" s="1">
+        <v>237.7</v>
+      </c>
+      <c r="F72" s="1">
+        <v>8.3</v>
+      </c>
+      <c r="G72" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H72" s="1">
+        <v>52.2</v>
+      </c>
+    </row>
+    <row r="73" customHeight="1" spans="1:8">
+      <c r="A73" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D73" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="E73" s="1">
+        <v>180.2</v>
+      </c>
+      <c r="F73" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="G73" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H73" s="1">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="74" customHeight="1" spans="1:8">
+      <c r="A74" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D74" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="E74" s="1">
+        <v>234</v>
+      </c>
+      <c r="F74" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="G74" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H74" s="1">
+        <v>49.9</v>
+      </c>
+    </row>
+    <row r="75" customHeight="1" spans="1:8">
+      <c r="A75" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D75" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="E75" s="1">
+        <v>214.6</v>
+      </c>
+      <c r="F75" s="1">
+        <v>-0.7</v>
+      </c>
+      <c r="G75" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H75" s="1">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="76" customHeight="1" spans="1:8">
+      <c r="A76" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D76" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="E76" s="1">
+        <v>223.8</v>
+      </c>
+      <c r="F76" s="1">
+        <v>-1</v>
+      </c>
+      <c r="G76" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H76" s="1">
+        <v>43.3</v>
+      </c>
+    </row>
+    <row r="77" customHeight="1" spans="1:8">
+      <c r="A77" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D77" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="E77" s="1">
+        <v>179.2</v>
+      </c>
+      <c r="F77" s="1">
+        <v>-1.7</v>
+      </c>
+      <c r="G77" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H77" s="1">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="78" customHeight="1" spans="1:8">
+      <c r="A78" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D78" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="E78" s="1">
+        <v>195.7</v>
+      </c>
+      <c r="F78" s="1">
+        <v>-2.1</v>
+      </c>
+      <c r="G78" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H78" s="1">
+        <v>25.3</v>
+      </c>
+    </row>
+    <row r="79" customHeight="1" spans="1:8">
+      <c r="A79" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D79" s="1">
+        <v>200</v>
+      </c>
+      <c r="E79" s="1">
+        <v>195</v>
+      </c>
+      <c r="F79" s="1">
+        <v>-2.5</v>
+      </c>
+      <c r="G79" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H79" s="1">
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="80" customHeight="1" spans="1:8">
+      <c r="A80" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D80" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="E80" s="1">
+        <v>174.3</v>
+      </c>
+      <c r="F80" s="1">
+        <v>-5.9</v>
+      </c>
+      <c r="G80" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H80" s="1">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="81" customHeight="1" spans="1:8">
+      <c r="A81" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D81" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="E81" s="1">
+        <v>173.4</v>
+      </c>
+      <c r="F81" s="1">
+        <v>-13.3</v>
+      </c>
+      <c r="G81" s="1">
+        <v>156.1</v>
+      </c>
+      <c r="H81" s="1">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="82" customHeight="1" spans="1:8">
+      <c r="A82" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D82" s="1">
+        <v>119.2</v>
+      </c>
+      <c r="E82" s="1">
+        <v>345.9</v>
+      </c>
+      <c r="F82" s="1">
+        <v>190.1</v>
+      </c>
+      <c r="G82" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H82" s="1">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="83" customHeight="1" spans="1:8">
+      <c r="A83" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D83" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="E83" s="1">
+        <v>148</v>
+      </c>
+      <c r="F83" s="1">
+        <v>20.8</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" customHeight="1" spans="1:8">
+      <c r="A84" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D84" s="1">
+        <v>130.7</v>
+      </c>
+      <c r="E84" s="1">
+        <v>156.5</v>
+      </c>
+      <c r="F84" s="1">
+        <v>19.7</v>
+      </c>
+      <c r="G84" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H84" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" customHeight="1" spans="1:8">
+      <c r="A85" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D85" s="1">
+        <v>133</v>
+      </c>
+      <c r="E85" s="1">
+        <v>158.2</v>
+      </c>
+      <c r="F85" s="1">
+        <v>18.9</v>
+      </c>
+      <c r="G85" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H85" s="1">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="86" customHeight="1" spans="1:8">
+      <c r="A86" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D86" s="1">
+        <v>100.7</v>
+      </c>
+      <c r="E86" s="1">
+        <v>115.7</v>
+      </c>
+      <c r="F86" s="1">
+        <v>14.8</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" customHeight="1" spans="1:8">
+      <c r="A87" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D87" s="1">
+        <v>154.1</v>
+      </c>
+      <c r="E87" s="1">
+        <v>176.6</v>
+      </c>
+      <c r="F87" s="1">
+        <v>14.5</v>
+      </c>
+      <c r="G87" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H87" s="1">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="88" customHeight="1" spans="1:8">
+      <c r="A88" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D88" s="1">
+        <v>88.7</v>
+      </c>
+      <c r="E88" s="1">
+        <v>101.5</v>
+      </c>
+      <c r="F88" s="1">
+        <v>14.4</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="89" customHeight="1" spans="1:8">
+      <c r="A89" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D89" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="E89" s="1">
+        <v>242.9</v>
+      </c>
+      <c r="F89" s="1">
+        <v>14.2</v>
+      </c>
+      <c r="G89" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H89" s="1">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="90" customHeight="1" spans="1:8">
+      <c r="A90" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="E90" s="1">
+        <v>118.5</v>
+      </c>
+      <c r="F90" s="1">
+        <v>14</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="91" customHeight="1" spans="1:8">
+      <c r="A91" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D91" s="1">
+        <v>149.4</v>
+      </c>
+      <c r="E91" s="1">
+        <v>167</v>
+      </c>
+      <c r="F91" s="1">
+        <v>11.7</v>
+      </c>
+      <c r="G91" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H91" s="1">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="92" customHeight="1" spans="1:8">
+      <c r="A92" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D92" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="E92" s="1">
+        <v>165.9</v>
+      </c>
+      <c r="F92" s="1">
+        <v>11.7</v>
+      </c>
+      <c r="G92" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H92" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="93" customHeight="1" spans="1:8">
+      <c r="A93" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D93" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="E93" s="1">
+        <v>110.9</v>
+      </c>
+      <c r="F93" s="1">
+        <v>11.5</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H93" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="94" customHeight="1" spans="1:8">
+      <c r="A94" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D94" s="1">
+        <v>113.9</v>
+      </c>
+      <c r="E94" s="1">
+        <v>126.9</v>
+      </c>
+      <c r="F94" s="1">
+        <v>11.4</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="95" customHeight="1" spans="1:8">
+      <c r="A95" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D95" s="1">
+        <v>95.5</v>
+      </c>
+      <c r="E95" s="1">
+        <v>105.7</v>
+      </c>
+      <c r="F95" s="1">
+        <v>10.6</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H95" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="96" customHeight="1" spans="1:8">
+      <c r="A96" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D96" s="1">
+        <v>107.6</v>
+      </c>
+      <c r="E96" s="1">
+        <v>118.9</v>
+      </c>
+      <c r="F96" s="1">
+        <v>10.4</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H96" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="97" customHeight="1" spans="1:8">
+      <c r="A97" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D97" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="E97" s="1">
+        <v>167.4</v>
+      </c>
+      <c r="F97" s="1">
+        <v>10.2</v>
+      </c>
+      <c r="G97" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H97" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="98" customHeight="1" spans="1:8">
+      <c r="A98" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D98" s="1">
+        <v>146.1</v>
+      </c>
+      <c r="E98" s="1">
+        <v>160.7</v>
+      </c>
+      <c r="F98" s="1">
+        <v>10</v>
+      </c>
+      <c r="G98" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H98" s="1">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="99" customHeight="1" spans="1:8">
+      <c r="A99" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D99" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="E99" s="1">
+        <v>205.3</v>
+      </c>
+      <c r="F99" s="1">
+        <v>9.6</v>
+      </c>
+      <c r="G99" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H99" s="1">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="100" customHeight="1" spans="1:8">
+      <c r="A100" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D100" s="1">
+        <v>169.8</v>
+      </c>
+      <c r="E100" s="1">
+        <v>185.7</v>
+      </c>
+      <c r="F100" s="1">
+        <v>9.3</v>
+      </c>
+      <c r="G100" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H100" s="1">
+        <v>18.6</v>
+      </c>
+    </row>
+    <row r="101" customHeight="1" spans="1:8">
+      <c r="A101" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D101" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="E101" s="1">
+        <v>239</v>
+      </c>
+      <c r="F101" s="1">
+        <v>8.9</v>
+      </c>
+      <c r="G101" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H101" s="1">
+        <v>52.7</v>
+      </c>
+    </row>
+    <row r="102" customHeight="1" spans="1:8">
+      <c r="A102" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D102" s="1">
+        <v>166</v>
+      </c>
+      <c r="E102" s="1">
+        <v>180.1</v>
+      </c>
+      <c r="F102" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="G102" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H102" s="1">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="103" customHeight="1" spans="1:8">
+      <c r="A103" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D103" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="E103" s="1">
+        <v>180.9</v>
+      </c>
+      <c r="F103" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="G103" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H103" s="1">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="104" customHeight="1" spans="1:8">
+      <c r="A104" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D104" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="E104" s="1">
+        <v>234.3</v>
+      </c>
+      <c r="F104" s="1">
+        <v>6.3</v>
+      </c>
+      <c r="G104" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H104" s="1">
+        <v>49.7</v>
+      </c>
+    </row>
+    <row r="105" customHeight="1" spans="1:8">
+      <c r="A105" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D105" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="E105" s="1">
+        <v>183.3</v>
+      </c>
+      <c r="F105" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G105" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H105" s="1">
+        <v>17.1</v>
+      </c>
+    </row>
+    <row r="106" customHeight="1" spans="1:8">
+      <c r="A106" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D106" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="E106" s="1">
+        <v>226.5</v>
+      </c>
+      <c r="F106" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G106" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H106" s="1">
+        <v>44.8</v>
+      </c>
+    </row>
+    <row r="107" customHeight="1" spans="1:8">
+      <c r="A107" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D107" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="E107" s="1">
+        <v>197.2</v>
+      </c>
+      <c r="F107" s="1">
+        <v>-1.3</v>
+      </c>
+      <c r="G107" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H107" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="108" customHeight="1" spans="1:8">
+      <c r="A108" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D108" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="E108" s="1">
+        <v>213.2</v>
+      </c>
+      <c r="F108" s="1">
+        <v>-1.3</v>
+      </c>
+      <c r="G108" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H108" s="1">
+        <v>36.3</v>
+      </c>
+    </row>
+    <row r="109" customHeight="1" spans="1:8">
+      <c r="A109" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D109" s="1">
+        <v>200</v>
+      </c>
+      <c r="E109" s="1">
+        <v>195.1</v>
+      </c>
+      <c r="F109" s="1">
+        <v>-2.4</v>
+      </c>
+      <c r="G109" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H109" s="1">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="110" customHeight="1" spans="1:8">
+      <c r="A110" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D110" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="E110" s="1">
+        <v>174.1</v>
+      </c>
+      <c r="F110" s="1">
+        <v>-6</v>
+      </c>
+      <c r="G110" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H110" s="1">
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="111" customHeight="1" spans="1:8">
+      <c r="A111" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D111" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="E111" s="1">
+        <v>175.8</v>
+      </c>
+      <c r="F111" s="1">
+        <v>-12.1</v>
+      </c>
+      <c r="G111" s="1">
+        <v>156.4</v>
+      </c>
+      <c r="H111" s="1">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="112" customHeight="1" spans="1:8">
+      <c r="A112" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D112" s="1">
+        <v>119.2</v>
+      </c>
+      <c r="E112" s="1">
+        <v>149</v>
+      </c>
+      <c r="F112" s="1">
+        <v>25</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H112" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="113" customHeight="1" spans="1:8">
+      <c r="A113" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D113" s="1">
+        <v>130.7</v>
+      </c>
+      <c r="E113" s="1">
+        <v>159.6</v>
+      </c>
+      <c r="F113" s="1">
+        <v>22</v>
+      </c>
+      <c r="G113" s="1">
+        <v>156</v>
+      </c>
+      <c r="H113" s="1">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="114" customHeight="1" spans="1:8">
+      <c r="A114" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D114" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="E114" s="1">
+        <v>148.6</v>
+      </c>
+      <c r="F114" s="1">
+        <v>21.3</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H114" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="115" customHeight="1" spans="1:8">
+      <c r="A115" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D115" s="1">
+        <v>133</v>
+      </c>
+      <c r="E115" s="1">
+        <v>154.9</v>
+      </c>
+      <c r="F115" s="1">
+        <v>16.4</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H115" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="116" customHeight="1" spans="1:8">
+      <c r="A116" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D116" s="1">
+        <v>100.7</v>
+      </c>
+      <c r="E116" s="1">
+        <v>114.9</v>
+      </c>
+      <c r="F116" s="1">
+        <v>14</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H116" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="117" customHeight="1" spans="1:8">
+      <c r="A117" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D117" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="E117" s="1">
+        <v>113.2</v>
+      </c>
+      <c r="F117" s="1">
+        <v>13.9</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H117" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="118" customHeight="1" spans="1:8">
+      <c r="A118" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D118" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="E118" s="1">
+        <v>118.3</v>
+      </c>
+      <c r="F118" s="1">
+        <v>13.8</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H118" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="119" customHeight="1" spans="1:8">
+      <c r="A119" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D119" s="1">
+        <v>154.1</v>
+      </c>
+      <c r="E119" s="1">
+        <v>175.3</v>
+      </c>
+      <c r="F119" s="1">
+        <v>13.7</v>
+      </c>
+      <c r="G119" s="1">
+        <v>156</v>
+      </c>
+      <c r="H119" s="1">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="120" customHeight="1" spans="1:8">
+      <c r="A120" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D120" s="1">
+        <v>88.7</v>
+      </c>
+      <c r="E120" s="1">
+        <v>100.8</v>
+      </c>
+      <c r="F120" s="1">
+        <v>13.5</v>
+      </c>
+      <c r="G120" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H120" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="121" customHeight="1" spans="1:8">
+      <c r="A121" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D121" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="E121" s="1">
+        <v>166.7</v>
+      </c>
+      <c r="F121" s="1">
+        <v>12.2</v>
+      </c>
+      <c r="G121" s="1">
+        <v>156</v>
+      </c>
+      <c r="H121" s="1">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="122" customHeight="1" spans="1:8">
+      <c r="A122" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D122" s="1">
+        <v>95.5</v>
+      </c>
+      <c r="E122" s="1">
+        <v>107</v>
+      </c>
+      <c r="F122" s="1">
+        <v>12</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="123" customHeight="1" spans="1:8">
+      <c r="A123" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D123" s="1">
+        <v>149.4</v>
+      </c>
+      <c r="E123" s="1">
+        <v>167.1</v>
+      </c>
+      <c r="F123" s="1">
+        <v>11.8</v>
+      </c>
+      <c r="G123" s="1">
+        <v>156</v>
+      </c>
+      <c r="H123" s="1">
+        <v>7.1</v>
+      </c>
+    </row>
+    <row r="124" customHeight="1" spans="1:8">
+      <c r="A124" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D124" s="1">
+        <v>113.9</v>
+      </c>
+      <c r="E124" s="1">
+        <v>127</v>
+      </c>
+      <c r="F124" s="1">
+        <v>11.4</v>
+      </c>
+      <c r="G124" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H124" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="125" customHeight="1" spans="1:8">
+      <c r="A125" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D125" s="1">
+        <v>146.1</v>
+      </c>
+      <c r="E125" s="1">
+        <v>161.2</v>
+      </c>
+      <c r="F125" s="1">
+        <v>10.3</v>
+      </c>
+      <c r="G125" s="1">
+        <v>156</v>
+      </c>
+      <c r="H125" s="1">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="126" customHeight="1" spans="1:8">
+      <c r="A126" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D126" s="1">
+        <v>169.8</v>
+      </c>
+      <c r="E126" s="1">
+        <v>186.8</v>
+      </c>
+      <c r="F126" s="1">
+        <v>10</v>
+      </c>
+      <c r="G126" s="1">
+        <v>156</v>
+      </c>
+      <c r="H126" s="1">
+        <v>19.7</v>
+      </c>
+    </row>
+    <row r="127" customHeight="1" spans="1:8">
+      <c r="A127" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D127" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="E127" s="1">
+        <v>204.8</v>
+      </c>
+      <c r="F127" s="1">
+        <v>9.3</v>
+      </c>
+      <c r="G127" s="1">
+        <v>156</v>
+      </c>
+      <c r="H127" s="1">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="128" customHeight="1" spans="1:8">
+      <c r="A128" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D128" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="E128" s="1">
+        <v>239.5</v>
+      </c>
+      <c r="F128" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="G128" s="1">
+        <v>156</v>
+      </c>
+      <c r="H128" s="1">
+        <v>53.4</v>
+      </c>
+    </row>
+    <row r="129" customHeight="1" spans="1:8">
+      <c r="A129" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D129" s="1">
+        <v>166</v>
+      </c>
+      <c r="E129" s="1">
+        <v>180.6</v>
+      </c>
+      <c r="F129" s="1">
+        <v>8.7</v>
+      </c>
+      <c r="G129" s="1">
+        <v>156</v>
+      </c>
+      <c r="H129" s="1">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="130" customHeight="1" spans="1:8">
+      <c r="A130" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D130" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="E130" s="1">
+        <v>231.1</v>
+      </c>
+      <c r="F130" s="1">
+        <v>8.6</v>
+      </c>
+      <c r="G130" s="1">
+        <v>156</v>
+      </c>
+      <c r="H130" s="1">
+        <v>48.1</v>
+      </c>
+    </row>
+    <row r="131" customHeight="1" spans="1:8">
+      <c r="A131" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D131" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="E131" s="1">
+        <v>181</v>
+      </c>
+      <c r="F131" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="G131" s="1">
+        <v>156</v>
+      </c>
+      <c r="H131" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="132" customHeight="1" spans="1:8">
+      <c r="A132" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D132" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="E132" s="1">
+        <v>235.1</v>
+      </c>
+      <c r="F132" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="G132" s="1">
+        <v>156</v>
+      </c>
+      <c r="H132" s="1">
+        <v>50.6</v>
+      </c>
+    </row>
+    <row r="133" customHeight="1" spans="1:8">
+      <c r="A133" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D133" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="E133" s="1">
+        <v>186</v>
+      </c>
+      <c r="F133" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="G133" s="1">
+        <v>156</v>
+      </c>
+      <c r="H133" s="1">
+        <v>19.2</v>
+      </c>
+    </row>
+    <row r="134" customHeight="1" spans="1:8">
+      <c r="A134" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D134" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="E134" s="1">
+        <v>224.7</v>
+      </c>
+      <c r="F134" s="1">
+        <v>-0.6</v>
+      </c>
+      <c r="G134" s="1">
+        <v>156</v>
+      </c>
+      <c r="H134" s="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="135" customHeight="1" spans="1:8">
+      <c r="A135" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D135" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="E135" s="1">
+        <v>214.8</v>
+      </c>
+      <c r="F135" s="1">
+        <v>-0.6</v>
+      </c>
+      <c r="G135" s="1">
+        <v>156</v>
+      </c>
+      <c r="H135" s="1">
+        <v>37.7</v>
+      </c>
+    </row>
+    <row r="136" customHeight="1" spans="1:8">
+      <c r="A136" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D136" s="1">
+        <v>200</v>
+      </c>
+      <c r="E136" s="1">
+        <v>195.9</v>
+      </c>
+      <c r="F136" s="1">
+        <v>-2</v>
+      </c>
+      <c r="G136" s="1">
+        <v>156</v>
+      </c>
+      <c r="H136" s="1">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="137" customHeight="1" spans="1:8">
+      <c r="A137" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D137" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="E137" s="1">
+        <v>195.7</v>
+      </c>
+      <c r="F137" s="1">
+        <v>-2.1</v>
+      </c>
+      <c r="G137" s="1">
+        <v>156</v>
+      </c>
+      <c r="H137" s="1">
+        <v>25.4</v>
+      </c>
+    </row>
+    <row r="138" customHeight="1" spans="1:8">
+      <c r="A138" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B138" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D138" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="E138" s="1">
+        <v>174.4</v>
+      </c>
+      <c r="F138" s="1">
+        <v>-5.9</v>
+      </c>
+      <c r="G138" s="1">
+        <v>156</v>
+      </c>
+      <c r="H138" s="1">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="139" customHeight="1" spans="1:8">
+      <c r="A139" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B139" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D139" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="E139" s="1">
+        <v>176.4</v>
+      </c>
+      <c r="F139" s="1">
+        <v>-11.8</v>
+      </c>
+      <c r="G139" s="1">
+        <v>156</v>
+      </c>
+      <c r="H139" s="1">
+        <v>13.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: 2026/06/16 周二 17:11:52.75
</commit_message>
<xml_diff>
--- a/source/8、绩效异常岗位/1、装车岗/装车岗-6月.xlsx
+++ b/source/8、绩效异常岗位/1、装车岗/装车岗-6月.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$H$219</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="86">
   <si>
     <t>岗位类型</t>
   </si>
@@ -272,6 +272,24 @@
   </si>
   <si>
     <t>2026-06-08</t>
+  </si>
+  <si>
+    <t>2026-06-09</t>
+  </si>
+  <si>
+    <t>2026-06-10</t>
+  </si>
+  <si>
+    <t>2026-06-11</t>
+  </si>
+  <si>
+    <t>2026-06-12</t>
+  </si>
+  <si>
+    <t>2026-06-13</t>
+  </si>
+  <si>
+    <t>2026-06-14</t>
   </si>
 </sst>
 </file>
@@ -1205,7 +1223,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I219"/>
+  <dimension ref="A1:I348"/>
   <sheetFormatPr defaultColWidth="12.6363636363636" defaultRowHeight="20" customHeight="1"/>
   <cols>
     <col min="1" max="16384" width="12.6363636363636" style="1" customWidth="1"/>
@@ -7562,8 +7580,3749 @@
         <v>14.3</v>
       </c>
     </row>
+    <row r="220" customHeight="1" spans="1:9">
+      <c r="A220" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C220" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D220" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E220" s="1">
+        <v>130.7</v>
+      </c>
+      <c r="F220" s="1">
+        <v>160.9</v>
+      </c>
+      <c r="G220" s="1">
+        <v>23</v>
+      </c>
+      <c r="H220" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I220" s="1">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="221" customHeight="1" spans="1:9">
+      <c r="A221" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C221" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D221" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E221" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="F221" s="1">
+        <v>146.1</v>
+      </c>
+      <c r="G221" s="1">
+        <v>19.3</v>
+      </c>
+      <c r="H221" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I221" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="222" customHeight="1" spans="1:9">
+      <c r="A222" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B222" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C222" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D222" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E222" s="1">
+        <v>126.9</v>
+      </c>
+      <c r="F222" s="1">
+        <v>151.4</v>
+      </c>
+      <c r="G222" s="1">
+        <v>19.3</v>
+      </c>
+      <c r="H222" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I222" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="223" customHeight="1" spans="1:9">
+      <c r="A223" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B223" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C223" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D223" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E223" s="1">
+        <v>133</v>
+      </c>
+      <c r="F223" s="1">
+        <v>151.5</v>
+      </c>
+      <c r="G223" s="1">
+        <v>13.8</v>
+      </c>
+      <c r="H223" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I223" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="224" customHeight="1" spans="1:9">
+      <c r="A224" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B224" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C224" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D224" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E224" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="F224" s="1">
+        <v>112</v>
+      </c>
+      <c r="G224" s="1">
+        <v>12.6</v>
+      </c>
+      <c r="H224" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I224" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="225" customHeight="1" spans="1:9">
+      <c r="A225" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B225" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C225" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D225" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E225" s="1">
+        <v>154.1</v>
+      </c>
+      <c r="F225" s="1">
+        <v>172.2</v>
+      </c>
+      <c r="G225" s="1">
+        <v>11.7</v>
+      </c>
+      <c r="H225" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I225" s="1">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="226" customHeight="1" spans="1:9">
+      <c r="A226" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B226" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C226" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D226" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E226" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="F226" s="1">
+        <v>116.1</v>
+      </c>
+      <c r="G226" s="1">
+        <v>11.6</v>
+      </c>
+      <c r="H226" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I226" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="227" customHeight="1" spans="1:9">
+      <c r="A227" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C227" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D227" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E227" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F227" s="1">
+        <v>165.7</v>
+      </c>
+      <c r="G227" s="1">
+        <v>11.6</v>
+      </c>
+      <c r="H227" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I227" s="1">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="228" customHeight="1" spans="1:9">
+      <c r="A228" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B228" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C228" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D228" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E228" s="1">
+        <v>100.7</v>
+      </c>
+      <c r="F228" s="1">
+        <v>112</v>
+      </c>
+      <c r="G228" s="1">
+        <v>11.1</v>
+      </c>
+      <c r="H228" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I228" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="229" customHeight="1" spans="1:9">
+      <c r="A229" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B229" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C229" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D229" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E229" s="1">
+        <v>149.4</v>
+      </c>
+      <c r="F229" s="1">
+        <v>165.3</v>
+      </c>
+      <c r="G229" s="1">
+        <v>10.6</v>
+      </c>
+      <c r="H229" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I229" s="1">
+        <v>8.3</v>
+      </c>
+    </row>
+    <row r="230" customHeight="1" spans="1:9">
+      <c r="A230" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C230" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D230" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E230" s="1">
+        <v>166</v>
+      </c>
+      <c r="F230" s="1">
+        <v>178.5</v>
+      </c>
+      <c r="G230" s="1">
+        <v>7.4</v>
+      </c>
+      <c r="H230" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I230" s="1">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="231" customHeight="1" spans="1:9">
+      <c r="A231" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C231" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D231" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E231" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="F231" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="G231" s="1">
+        <v>6.9</v>
+      </c>
+      <c r="H231" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I231" s="1">
+        <v>31.2</v>
+      </c>
+    </row>
+    <row r="232" customHeight="1" spans="1:9">
+      <c r="A232" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B232" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C232" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D232" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E232" s="1">
+        <v>169.8</v>
+      </c>
+      <c r="F232" s="1">
+        <v>181.4</v>
+      </c>
+      <c r="G232" s="1">
+        <v>6.8</v>
+      </c>
+      <c r="H232" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I232" s="1">
+        <v>18.8</v>
+      </c>
+    </row>
+    <row r="233" customHeight="1" spans="1:9">
+      <c r="A233" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B233" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C233" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D233" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E233" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="F233" s="1">
+        <v>232.3</v>
+      </c>
+      <c r="G233" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="H233" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I233" s="1">
+        <v>52.2</v>
+      </c>
+    </row>
+    <row r="234" customHeight="1" spans="1:9">
+      <c r="A234" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B234" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C234" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D234" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E234" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="F234" s="1">
+        <v>178.2</v>
+      </c>
+      <c r="G234" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="H234" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I234" s="1">
+        <v>16.8</v>
+      </c>
+    </row>
+    <row r="235" customHeight="1" spans="1:9">
+      <c r="A235" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B235" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C235" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D235" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E235" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="F235" s="1">
+        <v>229.7</v>
+      </c>
+      <c r="G235" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="H235" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I235" s="1">
+        <v>50.5</v>
+      </c>
+    </row>
+    <row r="236" customHeight="1" spans="1:9">
+      <c r="A236" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B236" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C236" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D236" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E236" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="F236" s="1">
+        <v>216.8</v>
+      </c>
+      <c r="G236" s="1">
+        <v>1.9</v>
+      </c>
+      <c r="H236" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I236" s="1">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="237" customHeight="1" spans="1:9">
+      <c r="A237" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C237" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D237" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E237" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="F237" s="1">
+        <v>181.6</v>
+      </c>
+      <c r="G237" s="1">
+        <v>-0.4</v>
+      </c>
+      <c r="H237" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I237" s="1">
+        <v>18.9</v>
+      </c>
+    </row>
+    <row r="238" customHeight="1" spans="1:9">
+      <c r="A238" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C238" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D238" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E238" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="F238" s="1">
+        <v>197.5</v>
+      </c>
+      <c r="G238" s="1">
+        <v>-1.2</v>
+      </c>
+      <c r="H238" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I238" s="1">
+        <v>29.4</v>
+      </c>
+    </row>
+    <row r="239" customHeight="1" spans="1:9">
+      <c r="A239" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B239" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C239" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D239" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E239" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="F239" s="1">
+        <v>220.8</v>
+      </c>
+      <c r="G239" s="1">
+        <v>-2.3</v>
+      </c>
+      <c r="H239" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I239" s="1">
+        <v>44.6</v>
+      </c>
+    </row>
+    <row r="240" customHeight="1" spans="1:9">
+      <c r="A240" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B240" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C240" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D240" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E240" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="F240" s="1">
+        <v>209.5</v>
+      </c>
+      <c r="G240" s="1">
+        <v>-3</v>
+      </c>
+      <c r="H240" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I240" s="1">
+        <v>37.2</v>
+      </c>
+    </row>
+    <row r="241" customHeight="1" spans="1:9">
+      <c r="A241" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B241" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C241" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D241" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E241" s="1">
+        <v>200</v>
+      </c>
+      <c r="F241" s="1">
+        <v>189.3</v>
+      </c>
+      <c r="G241" s="1">
+        <v>-5.3</v>
+      </c>
+      <c r="H241" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I241" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="242" customHeight="1" spans="1:9">
+      <c r="A242" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B242" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C242" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D242" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E242" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="F242" s="1">
+        <v>171.1</v>
+      </c>
+      <c r="G242" s="1">
+        <v>-7.7</v>
+      </c>
+      <c r="H242" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I242" s="1">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="243" customHeight="1" spans="1:9">
+      <c r="A243" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C243" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D243" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E243" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="F243" s="1">
+        <v>176.1</v>
+      </c>
+      <c r="G243" s="1">
+        <v>-12</v>
+      </c>
+      <c r="H243" s="1">
+        <v>152.6</v>
+      </c>
+      <c r="I243" s="1">
+        <v>15.3</v>
+      </c>
+    </row>
+    <row r="244" customHeight="1" spans="1:9">
+      <c r="A244" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C244" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D244" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E244" s="1">
+        <v>130.7</v>
+      </c>
+      <c r="F244" s="1">
+        <v>160.2</v>
+      </c>
+      <c r="G244" s="1">
+        <v>22.5</v>
+      </c>
+      <c r="H244" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I244" s="1">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="245" customHeight="1" spans="1:9">
+      <c r="A245" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C245" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D245" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E245" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="F245" s="1">
+        <v>146.3</v>
+      </c>
+      <c r="G245" s="1">
+        <v>19.4</v>
+      </c>
+      <c r="H245" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I245" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="246" customHeight="1" spans="1:9">
+      <c r="A246" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C246" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D246" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E246" s="1">
+        <v>126.9</v>
+      </c>
+      <c r="F246" s="1">
+        <v>147.1</v>
+      </c>
+      <c r="G246" s="1">
+        <v>15.9</v>
+      </c>
+      <c r="H246" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I246" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="247" customHeight="1" spans="1:9">
+      <c r="A247" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C247" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D247" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E247" s="1">
+        <v>133</v>
+      </c>
+      <c r="F247" s="1">
+        <v>151</v>
+      </c>
+      <c r="G247" s="1">
+        <v>13.5</v>
+      </c>
+      <c r="H247" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I247" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="248" customHeight="1" spans="1:9">
+      <c r="A248" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C248" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D248" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E248" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="F248" s="1">
+        <v>112.1</v>
+      </c>
+      <c r="G248" s="1">
+        <v>12.8</v>
+      </c>
+      <c r="H248" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I248" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="249" customHeight="1" spans="1:9">
+      <c r="A249" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C249" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D249" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E249" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F249" s="1">
+        <v>165.3</v>
+      </c>
+      <c r="G249" s="1">
+        <v>11.3</v>
+      </c>
+      <c r="H249" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I249" s="1">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="250" customHeight="1" spans="1:9">
+      <c r="A250" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C250" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D250" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E250" s="1">
+        <v>154.1</v>
+      </c>
+      <c r="F250" s="1">
+        <v>171.5</v>
+      </c>
+      <c r="G250" s="1">
+        <v>11.2</v>
+      </c>
+      <c r="H250" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I250" s="1">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="251" customHeight="1" spans="1:9">
+      <c r="A251" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C251" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D251" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E251" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="F251" s="1">
+        <v>115.5</v>
+      </c>
+      <c r="G251" s="1">
+        <v>11.1</v>
+      </c>
+      <c r="H251" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I251" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="252" customHeight="1" spans="1:9">
+      <c r="A252" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C252" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D252" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E252" s="1">
+        <v>149.4</v>
+      </c>
+      <c r="F252" s="1">
+        <v>165.2</v>
+      </c>
+      <c r="G252" s="1">
+        <v>10.5</v>
+      </c>
+      <c r="H252" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I252" s="1">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="253" customHeight="1" spans="1:9">
+      <c r="A253" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C253" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D253" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E253" s="1">
+        <v>100.7</v>
+      </c>
+      <c r="F253" s="1">
+        <v>111.2</v>
+      </c>
+      <c r="G253" s="1">
+        <v>10.4</v>
+      </c>
+      <c r="H253" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I253" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="254" customHeight="1" spans="1:9">
+      <c r="A254" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C254" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D254" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E254" s="1">
+        <v>166</v>
+      </c>
+      <c r="F254" s="1">
+        <v>178.8</v>
+      </c>
+      <c r="G254" s="1">
+        <v>7.7</v>
+      </c>
+      <c r="H254" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I254" s="1">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="255" customHeight="1" spans="1:9">
+      <c r="A255" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C255" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D255" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E255" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="F255" s="1">
+        <v>199.7</v>
+      </c>
+      <c r="G255" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="H255" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I255" s="1">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="256" customHeight="1" spans="1:9">
+      <c r="A256" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C256" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D256" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E256" s="1">
+        <v>169.8</v>
+      </c>
+      <c r="F256" s="1">
+        <v>180.8</v>
+      </c>
+      <c r="G256" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="H256" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I256" s="1">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="257" customHeight="1" spans="1:9">
+      <c r="A257" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C257" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D257" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E257" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="F257" s="1">
+        <v>232.9</v>
+      </c>
+      <c r="G257" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="H257" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I257" s="1">
+        <v>52.8</v>
+      </c>
+    </row>
+    <row r="258" customHeight="1" spans="1:9">
+      <c r="A258" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C258" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D258" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E258" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="F258" s="1">
+        <v>178</v>
+      </c>
+      <c r="G258" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="H258" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I258" s="1">
+        <v>16.8</v>
+      </c>
+    </row>
+    <row r="259" customHeight="1" spans="1:9">
+      <c r="A259" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C259" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D259" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E259" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="F259" s="1">
+        <v>229.7</v>
+      </c>
+      <c r="G259" s="1">
+        <v>4.2</v>
+      </c>
+      <c r="H259" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I259" s="1">
+        <v>50.8</v>
+      </c>
+    </row>
+    <row r="260" customHeight="1" spans="1:9">
+      <c r="A260" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C260" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D260" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E260" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="F260" s="1">
+        <v>217.4</v>
+      </c>
+      <c r="G260" s="1">
+        <v>2.2</v>
+      </c>
+      <c r="H260" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I260" s="1">
+        <v>42.7</v>
+      </c>
+    </row>
+    <row r="261" customHeight="1" spans="1:9">
+      <c r="A261" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C261" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D261" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E261" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="F261" s="1">
+        <v>180.8</v>
+      </c>
+      <c r="G261" s="1">
+        <v>-0.8</v>
+      </c>
+      <c r="H261" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I261" s="1">
+        <v>18.7</v>
+      </c>
+    </row>
+    <row r="262" customHeight="1" spans="1:9">
+      <c r="A262" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C262" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D262" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E262" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="F262" s="1">
+        <v>197.1</v>
+      </c>
+      <c r="G262" s="1">
+        <v>-1.4</v>
+      </c>
+      <c r="H262" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I262" s="1">
+        <v>29.4</v>
+      </c>
+    </row>
+    <row r="263" customHeight="1" spans="1:9">
+      <c r="A263" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B263" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C263" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D263" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E263" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="F263" s="1">
+        <v>220</v>
+      </c>
+      <c r="G263" s="1">
+        <v>-2.7</v>
+      </c>
+      <c r="H263" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I263" s="1">
+        <v>44.4</v>
+      </c>
+    </row>
+    <row r="264" customHeight="1" spans="1:9">
+      <c r="A264" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B264" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C264" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D264" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E264" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="F264" s="1">
+        <v>209</v>
+      </c>
+      <c r="G264" s="1">
+        <v>-3.2</v>
+      </c>
+      <c r="H264" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I264" s="1">
+        <v>37.2</v>
+      </c>
+    </row>
+    <row r="265" customHeight="1" spans="1:9">
+      <c r="A265" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C265" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D265" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E265" s="1">
+        <v>200</v>
+      </c>
+      <c r="F265" s="1">
+        <v>189</v>
+      </c>
+      <c r="G265" s="1">
+        <v>-5.4</v>
+      </c>
+      <c r="H265" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I265" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="266" customHeight="1" spans="1:9">
+      <c r="A266" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C266" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D266" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E266" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="F266" s="1">
+        <v>171.5</v>
+      </c>
+      <c r="G266" s="1">
+        <v>-7.4</v>
+      </c>
+      <c r="H266" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I266" s="1">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="267" customHeight="1" spans="1:9">
+      <c r="A267" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C267" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D267" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E267" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="F267" s="1">
+        <v>176.4</v>
+      </c>
+      <c r="G267" s="1">
+        <v>-11.9</v>
+      </c>
+      <c r="H267" s="1">
+        <v>152.3</v>
+      </c>
+      <c r="I267" s="1">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="268" customHeight="1" spans="1:9">
+      <c r="A268" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C268" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D268" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E268" s="1">
+        <v>130.7</v>
+      </c>
+      <c r="F268" s="1">
+        <v>159.4</v>
+      </c>
+      <c r="G268" s="1">
+        <v>21.9</v>
+      </c>
+      <c r="H268" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I268" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="269" customHeight="1" spans="1:9">
+      <c r="A269" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B269" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C269" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D269" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E269" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="F269" s="1">
+        <v>146.1</v>
+      </c>
+      <c r="G269" s="1">
+        <v>19.3</v>
+      </c>
+      <c r="H269" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I269" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="270" customHeight="1" spans="1:9">
+      <c r="A270" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B270" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C270" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D270" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E270" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F270" s="1">
+        <v>171.4</v>
+      </c>
+      <c r="G270" s="1">
+        <v>15.4</v>
+      </c>
+      <c r="H270" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I270" s="1">
+        <v>12.4</v>
+      </c>
+    </row>
+    <row r="271" customHeight="1" spans="1:9">
+      <c r="A271" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B271" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C271" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D271" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E271" s="1">
+        <v>126.9</v>
+      </c>
+      <c r="F271" s="1">
+        <v>144.4</v>
+      </c>
+      <c r="G271" s="1">
+        <v>13.8</v>
+      </c>
+      <c r="H271" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I271" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="272" customHeight="1" spans="1:9">
+      <c r="A272" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B272" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C272" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D272" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E272" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="F272" s="1">
+        <v>112.2</v>
+      </c>
+      <c r="G272" s="1">
+        <v>12.8</v>
+      </c>
+      <c r="H272" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I272" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="273" customHeight="1" spans="1:9">
+      <c r="A273" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B273" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C273" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D273" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E273" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F273" s="1">
+        <v>165.4</v>
+      </c>
+      <c r="G273" s="1">
+        <v>11.4</v>
+      </c>
+      <c r="H273" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I273" s="1">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="274" customHeight="1" spans="1:9">
+      <c r="A274" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B274" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C274" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D274" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E274" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="F274" s="1">
+        <v>115.4</v>
+      </c>
+      <c r="G274" s="1">
+        <v>11</v>
+      </c>
+      <c r="H274" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I274" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="275" customHeight="1" spans="1:9">
+      <c r="A275" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B275" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C275" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D275" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E275" s="1">
+        <v>149.4</v>
+      </c>
+      <c r="F275" s="1">
+        <v>164.9</v>
+      </c>
+      <c r="G275" s="1">
+        <v>10.3</v>
+      </c>
+      <c r="H275" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I275" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="276" customHeight="1" spans="1:9">
+      <c r="A276" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B276" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C276" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D276" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E276" s="1">
+        <v>100.7</v>
+      </c>
+      <c r="F276" s="1">
+        <v>111</v>
+      </c>
+      <c r="G276" s="1">
+        <v>10.1</v>
+      </c>
+      <c r="H276" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I276" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="277" customHeight="1" spans="1:9">
+      <c r="A277" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C277" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D277" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E277" s="1">
+        <v>166</v>
+      </c>
+      <c r="F277" s="1">
+        <v>179.6</v>
+      </c>
+      <c r="G277" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="H277" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I277" s="1">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="278" customHeight="1" spans="1:9">
+      <c r="A278" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C278" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D278" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E278" s="1">
+        <v>169.8</v>
+      </c>
+      <c r="F278" s="1">
+        <v>181.3</v>
+      </c>
+      <c r="G278" s="1">
+        <v>6.8</v>
+      </c>
+      <c r="H278" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I278" s="1">
+        <v>18.9</v>
+      </c>
+    </row>
+    <row r="279" customHeight="1" spans="1:9">
+      <c r="A279" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B279" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C279" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D279" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E279" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="F279" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="G279" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="H279" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I279" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="280" customHeight="1" spans="1:9">
+      <c r="A280" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C280" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D280" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E280" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="F280" s="1">
+        <v>233.4</v>
+      </c>
+      <c r="G280" s="1">
+        <v>6.4</v>
+      </c>
+      <c r="H280" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I280" s="1">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="281" customHeight="1" spans="1:9">
+      <c r="A281" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C281" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D281" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E281" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="F281" s="1">
+        <v>177.8</v>
+      </c>
+      <c r="G281" s="1">
+        <v>5.3</v>
+      </c>
+      <c r="H281" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I281" s="1">
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="282" customHeight="1" spans="1:9">
+      <c r="A282" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B282" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C282" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D282" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E282" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="F282" s="1">
+        <v>228.4</v>
+      </c>
+      <c r="G282" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="H282" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I282" s="1">
+        <v>49.7</v>
+      </c>
+    </row>
+    <row r="283" customHeight="1" spans="1:9">
+      <c r="A283" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B283" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C283" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D283" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E283" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="F283" s="1">
+        <v>216.9</v>
+      </c>
+      <c r="G283" s="1">
+        <v>2</v>
+      </c>
+      <c r="H283" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I283" s="1">
+        <v>42.2</v>
+      </c>
+    </row>
+    <row r="284" customHeight="1" spans="1:9">
+      <c r="A284" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B284" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C284" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D284" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E284" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="F284" s="1">
+        <v>198.5</v>
+      </c>
+      <c r="G284" s="1">
+        <v>-0.7</v>
+      </c>
+      <c r="H284" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I284" s="1">
+        <v>30.1</v>
+      </c>
+    </row>
+    <row r="285" customHeight="1" spans="1:9">
+      <c r="A285" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B285" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C285" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D285" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E285" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="F285" s="1">
+        <v>180.8</v>
+      </c>
+      <c r="G285" s="1">
+        <v>-0.8</v>
+      </c>
+      <c r="H285" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I285" s="1">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="286" customHeight="1" spans="1:9">
+      <c r="A286" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C286" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D286" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E286" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="F286" s="1">
+        <v>219.5</v>
+      </c>
+      <c r="G286" s="1">
+        <v>-2.9</v>
+      </c>
+      <c r="H286" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I286" s="1">
+        <v>43.9</v>
+      </c>
+    </row>
+    <row r="287" customHeight="1" spans="1:9">
+      <c r="A287" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B287" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C287" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D287" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E287" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="F287" s="1">
+        <v>208.9</v>
+      </c>
+      <c r="G287" s="1">
+        <v>-3.3</v>
+      </c>
+      <c r="H287" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I287" s="1">
+        <v>36.9</v>
+      </c>
+    </row>
+    <row r="288" customHeight="1" spans="1:9">
+      <c r="A288" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B288" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C288" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D288" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E288" s="1">
+        <v>200</v>
+      </c>
+      <c r="F288" s="1">
+        <v>188.4</v>
+      </c>
+      <c r="G288" s="1">
+        <v>-5.7</v>
+      </c>
+      <c r="H288" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I288" s="1">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="289" customHeight="1" spans="1:9">
+      <c r="A289" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B289" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C289" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D289" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E289" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="F289" s="1">
+        <v>173.1</v>
+      </c>
+      <c r="G289" s="1">
+        <v>-6.6</v>
+      </c>
+      <c r="H289" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I289" s="1">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="290" customHeight="1" spans="1:9">
+      <c r="A290" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B290" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C290" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D290" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E290" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="F290" s="1">
+        <v>177.1</v>
+      </c>
+      <c r="G290" s="1">
+        <v>-11.5</v>
+      </c>
+      <c r="H290" s="1">
+        <v>152.5</v>
+      </c>
+      <c r="I290" s="1">
+        <v>16.1</v>
+      </c>
+    </row>
+    <row r="291" customHeight="1" spans="1:9">
+      <c r="A291" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B291" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C291" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D291" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E291" s="1">
+        <v>122.5</v>
+      </c>
+      <c r="F291" s="1">
+        <v>146.4</v>
+      </c>
+      <c r="G291" s="1">
+        <v>19.5</v>
+      </c>
+      <c r="H291" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I291" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="292" customHeight="1" spans="1:9">
+      <c r="A292" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B292" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C292" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D292" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E292" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F292" s="1">
+        <v>170.4</v>
+      </c>
+      <c r="G292" s="1">
+        <v>14.7</v>
+      </c>
+      <c r="H292" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I292" s="1">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="293" customHeight="1" spans="1:9">
+      <c r="A293" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B293" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C293" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D293" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E293" s="1">
+        <v>139.7</v>
+      </c>
+      <c r="F293" s="1">
+        <v>159.1</v>
+      </c>
+      <c r="G293" s="1">
+        <v>13.9</v>
+      </c>
+      <c r="H293" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I293" s="1">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="294" customHeight="1" spans="1:9">
+      <c r="A294" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B294" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C294" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D294" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E294" s="1">
+        <v>159.4</v>
+      </c>
+      <c r="F294" s="1">
+        <v>180.7</v>
+      </c>
+      <c r="G294" s="1">
+        <v>13.3</v>
+      </c>
+      <c r="H294" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I294" s="1">
+        <v>18.6</v>
+      </c>
+    </row>
+    <row r="295" customHeight="1" spans="1:9">
+      <c r="A295" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B295" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C295" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D295" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E295" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="F295" s="1">
+        <v>111.9</v>
+      </c>
+      <c r="G295" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="H295" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I295" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="296" customHeight="1" spans="1:9">
+      <c r="A296" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B296" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C296" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D296" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E296" s="1">
+        <v>126.9</v>
+      </c>
+      <c r="F296" s="1">
+        <v>141.6</v>
+      </c>
+      <c r="G296" s="1">
+        <v>11.6</v>
+      </c>
+      <c r="H296" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I296" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="297" customHeight="1" spans="1:9">
+      <c r="A297" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B297" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C297" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D297" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E297" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F297" s="1">
+        <v>164.6</v>
+      </c>
+      <c r="G297" s="1">
+        <v>10.8</v>
+      </c>
+      <c r="H297" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I297" s="1">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="298" customHeight="1" spans="1:9">
+      <c r="A298" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B298" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C298" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D298" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E298" s="1">
+        <v>103.9</v>
+      </c>
+      <c r="F298" s="1">
+        <v>115</v>
+      </c>
+      <c r="G298" s="1">
+        <v>10.6</v>
+      </c>
+      <c r="H298" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I298" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="299" customHeight="1" spans="1:9">
+      <c r="A299" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B299" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C299" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D299" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E299" s="1">
+        <v>166</v>
+      </c>
+      <c r="F299" s="1">
+        <v>181.8</v>
+      </c>
+      <c r="G299" s="1">
+        <v>9.5</v>
+      </c>
+      <c r="H299" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I299" s="1">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="300" customHeight="1" spans="1:9">
+      <c r="A300" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B300" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C300" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D300" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E300" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="F300" s="1">
+        <v>234</v>
+      </c>
+      <c r="G300" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="H300" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I300" s="1">
+        <v>53.6</v>
+      </c>
+    </row>
+    <row r="301" customHeight="1" spans="1:9">
+      <c r="A301" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C301" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D301" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E301" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="F301" s="1">
+        <v>199.4</v>
+      </c>
+      <c r="G301" s="1">
+        <v>6.4</v>
+      </c>
+      <c r="H301" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I301" s="1">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="302" customHeight="1" spans="1:9">
+      <c r="A302" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C302" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D302" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E302" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="F302" s="1">
+        <v>177.3</v>
+      </c>
+      <c r="G302" s="1">
+        <v>5.1</v>
+      </c>
+      <c r="H302" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I302" s="1">
+        <v>16.4</v>
+      </c>
+    </row>
+    <row r="303" customHeight="1" spans="1:9">
+      <c r="A303" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B303" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C303" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D303" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E303" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="F303" s="1">
+        <v>228.5</v>
+      </c>
+      <c r="G303" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="H303" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I303" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="304" customHeight="1" spans="1:9">
+      <c r="A304" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C304" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D304" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E304" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="F304" s="1">
+        <v>217.5</v>
+      </c>
+      <c r="G304" s="1">
+        <v>2.2</v>
+      </c>
+      <c r="H304" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I304" s="1">
+        <v>42.8</v>
+      </c>
+    </row>
+    <row r="305" customHeight="1" spans="1:9">
+      <c r="A305" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C305" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D305" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E305" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="F305" s="1">
+        <v>198.6</v>
+      </c>
+      <c r="G305" s="1">
+        <v>-0.6</v>
+      </c>
+      <c r="H305" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I305" s="1">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="306" customHeight="1" spans="1:9">
+      <c r="A306" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B306" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C306" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D306" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E306" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="F306" s="1">
+        <v>180.6</v>
+      </c>
+      <c r="G306" s="1">
+        <v>-0.9</v>
+      </c>
+      <c r="H306" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I306" s="1">
+        <v>18.6</v>
+      </c>
+    </row>
+    <row r="307" customHeight="1" spans="1:9">
+      <c r="A307" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C307" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D307" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E307" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="F307" s="1">
+        <v>218.7</v>
+      </c>
+      <c r="G307" s="1">
+        <v>-3.2</v>
+      </c>
+      <c r="H307" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I307" s="1">
+        <v>43.6</v>
+      </c>
+    </row>
+    <row r="308" customHeight="1" spans="1:9">
+      <c r="A308" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C308" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D308" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E308" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="F308" s="1">
+        <v>207.9</v>
+      </c>
+      <c r="G308" s="1">
+        <v>-3.8</v>
+      </c>
+      <c r="H308" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I308" s="1">
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="309" customHeight="1" spans="1:9">
+      <c r="A309" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C309" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D309" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E309" s="1">
+        <v>200</v>
+      </c>
+      <c r="F309" s="1">
+        <v>188.3</v>
+      </c>
+      <c r="G309" s="1">
+        <v>-5.8</v>
+      </c>
+      <c r="H309" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I309" s="1">
+        <v>23.6</v>
+      </c>
+    </row>
+    <row r="310" customHeight="1" spans="1:9">
+      <c r="A310" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C310" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D310" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E310" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="F310" s="1">
+        <v>173.6</v>
+      </c>
+      <c r="G310" s="1">
+        <v>-6.3</v>
+      </c>
+      <c r="H310" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I310" s="1">
+        <v>13.9</v>
+      </c>
+    </row>
+    <row r="311" customHeight="1" spans="1:9">
+      <c r="A311" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B311" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C311" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D311" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E311" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="F311" s="1">
+        <v>177.9</v>
+      </c>
+      <c r="G311" s="1">
+        <v>-11.1</v>
+      </c>
+      <c r="H311" s="1">
+        <v>152.2</v>
+      </c>
+      <c r="I311" s="1">
+        <v>16.8</v>
+      </c>
+    </row>
+    <row r="312" customHeight="1" spans="1:9">
+      <c r="A312" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C312" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D312" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E312" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F312" s="1">
+        <v>170</v>
+      </c>
+      <c r="G312" s="1">
+        <v>14.5</v>
+      </c>
+      <c r="H312" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I312" s="1">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="313" customHeight="1" spans="1:9">
+      <c r="A313" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B313" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C313" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D313" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E313" s="1">
+        <v>139.7</v>
+      </c>
+      <c r="F313" s="1">
+        <v>158.5</v>
+      </c>
+      <c r="G313" s="1">
+        <v>13.4</v>
+      </c>
+      <c r="H313" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I313" s="1">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="314" customHeight="1" spans="1:9">
+      <c r="A314" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C314" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D314" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E314" s="1">
+        <v>159.4</v>
+      </c>
+      <c r="F314" s="1">
+        <v>179.8</v>
+      </c>
+      <c r="G314" s="1">
+        <v>12.8</v>
+      </c>
+      <c r="H314" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I314" s="1">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="315" customHeight="1" spans="1:9">
+      <c r="A315" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C315" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D315" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E315" s="1">
+        <v>126.9</v>
+      </c>
+      <c r="F315" s="1">
+        <v>142.7</v>
+      </c>
+      <c r="G315" s="1">
+        <v>12.4</v>
+      </c>
+      <c r="H315" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I315" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="316" customHeight="1" spans="1:9">
+      <c r="A316" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C316" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D316" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E316" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="F316" s="1">
+        <v>111.7</v>
+      </c>
+      <c r="G316" s="1">
+        <v>12.3</v>
+      </c>
+      <c r="H316" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I316" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="317" customHeight="1" spans="1:9">
+      <c r="A317" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B317" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C317" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D317" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E317" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F317" s="1">
+        <v>164.6</v>
+      </c>
+      <c r="G317" s="1">
+        <v>10.8</v>
+      </c>
+      <c r="H317" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I317" s="1">
+        <v>8.3</v>
+      </c>
+    </row>
+    <row r="318" customHeight="1" spans="1:9">
+      <c r="A318" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B318" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C318" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D318" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E318" s="1">
+        <v>166</v>
+      </c>
+      <c r="F318" s="1">
+        <v>183.4</v>
+      </c>
+      <c r="G318" s="1">
+        <v>10.4</v>
+      </c>
+      <c r="H318" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I318" s="1">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="319" customHeight="1" spans="1:9">
+      <c r="A319" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B319" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C319" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D319" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E319" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="F319" s="1">
+        <v>234</v>
+      </c>
+      <c r="G319" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="H319" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I319" s="1">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="320" customHeight="1" spans="1:9">
+      <c r="A320" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B320" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C320" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D320" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E320" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="F320" s="1">
+        <v>199.1</v>
+      </c>
+      <c r="G320" s="1">
+        <v>6.3</v>
+      </c>
+      <c r="H320" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I320" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="321" customHeight="1" spans="1:9">
+      <c r="A321" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B321" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C321" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D321" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E321" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="F321" s="1">
+        <v>176.8</v>
+      </c>
+      <c r="G321" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="H321" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I321" s="1">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="322" customHeight="1" spans="1:9">
+      <c r="A322" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C322" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D322" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E322" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="F322" s="1">
+        <v>227.9</v>
+      </c>
+      <c r="G322" s="1">
+        <v>3.4</v>
+      </c>
+      <c r="H322" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I322" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="323" customHeight="1" spans="1:9">
+      <c r="A323" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B323" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C323" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D323" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E323" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="F323" s="1">
+        <v>217.5</v>
+      </c>
+      <c r="G323" s="1">
+        <v>2.2</v>
+      </c>
+      <c r="H323" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I323" s="1">
+        <v>43.1</v>
+      </c>
+    </row>
+    <row r="324" customHeight="1" spans="1:9">
+      <c r="A324" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B324" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C324" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D324" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E324" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="F324" s="1">
+        <v>198.3</v>
+      </c>
+      <c r="G324" s="1">
+        <v>-0.8</v>
+      </c>
+      <c r="H324" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I324" s="1">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="325" customHeight="1" spans="1:9">
+      <c r="A325" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B325" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C325" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D325" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E325" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="F325" s="1">
+        <v>180.2</v>
+      </c>
+      <c r="G325" s="1">
+        <v>-1.2</v>
+      </c>
+      <c r="H325" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I325" s="1">
+        <v>18.6</v>
+      </c>
+    </row>
+    <row r="326" customHeight="1" spans="1:9">
+      <c r="A326" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C326" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D326" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E326" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="F326" s="1">
+        <v>217.8</v>
+      </c>
+      <c r="G326" s="1">
+        <v>-3.6</v>
+      </c>
+      <c r="H326" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I326" s="1">
+        <v>43.3</v>
+      </c>
+    </row>
+    <row r="327" customHeight="1" spans="1:9">
+      <c r="A327" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C327" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D327" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E327" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="F327" s="1">
+        <v>207</v>
+      </c>
+      <c r="G327" s="1">
+        <v>-4.2</v>
+      </c>
+      <c r="H327" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I327" s="1">
+        <v>36.2</v>
+      </c>
+    </row>
+    <row r="328" customHeight="1" spans="1:9">
+      <c r="A328" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B328" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C328" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D328" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E328" s="1">
+        <v>200</v>
+      </c>
+      <c r="F328" s="1">
+        <v>188.2</v>
+      </c>
+      <c r="G328" s="1">
+        <v>-5.8</v>
+      </c>
+      <c r="H328" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I328" s="1">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="329" customHeight="1" spans="1:9">
+      <c r="A329" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C329" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D329" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E329" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="F329" s="1">
+        <v>173.8</v>
+      </c>
+      <c r="G329" s="1">
+        <v>-6.2</v>
+      </c>
+      <c r="H329" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I329" s="1">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="330" customHeight="1" spans="1:9">
+      <c r="A330" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C330" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D330" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E330" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="F330" s="1">
+        <v>177.8</v>
+      </c>
+      <c r="G330" s="1">
+        <v>-11.1</v>
+      </c>
+      <c r="H330" s="1">
+        <v>151.9</v>
+      </c>
+      <c r="I330" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="331" customHeight="1" spans="1:9">
+      <c r="A331" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C331" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D331" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E331" s="1">
+        <v>148.5</v>
+      </c>
+      <c r="F331" s="1">
+        <v>170.2</v>
+      </c>
+      <c r="G331" s="1">
+        <v>14.6</v>
+      </c>
+      <c r="H331" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I331" s="1">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="332" customHeight="1" spans="1:9">
+      <c r="A332" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C332" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D332" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E332" s="1">
+        <v>126.9</v>
+      </c>
+      <c r="F332" s="1">
+        <v>143.8</v>
+      </c>
+      <c r="G332" s="1">
+        <v>13.3</v>
+      </c>
+      <c r="H332" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I332" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="333" customHeight="1" spans="1:9">
+      <c r="A333" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C333" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D333" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E333" s="1">
+        <v>139.7</v>
+      </c>
+      <c r="F333" s="1">
+        <v>158.2</v>
+      </c>
+      <c r="G333" s="1">
+        <v>13.2</v>
+      </c>
+      <c r="H333" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I333" s="1">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="334" customHeight="1" spans="1:9">
+      <c r="A334" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C334" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D334" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E334" s="1">
+        <v>99.4</v>
+      </c>
+      <c r="F334" s="1">
+        <v>111.5</v>
+      </c>
+      <c r="G334" s="1">
+        <v>12.1</v>
+      </c>
+      <c r="H334" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I334" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="335" customHeight="1" spans="1:9">
+      <c r="A335" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C335" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D335" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E335" s="1">
+        <v>166</v>
+      </c>
+      <c r="F335" s="1">
+        <v>183.4</v>
+      </c>
+      <c r="G335" s="1">
+        <v>10.4</v>
+      </c>
+      <c r="H335" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I335" s="1">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="336" customHeight="1" spans="1:9">
+      <c r="A336" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C336" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D336" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E336" s="1">
+        <v>219.3</v>
+      </c>
+      <c r="F336" s="1">
+        <v>235.9</v>
+      </c>
+      <c r="G336" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="H336" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I336" s="1">
+        <v>55.4</v>
+      </c>
+    </row>
+    <row r="337" customHeight="1" spans="1:9">
+      <c r="A337" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C337" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D337" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E337" s="1">
+        <v>187.3</v>
+      </c>
+      <c r="F337" s="1">
+        <v>198.8</v>
+      </c>
+      <c r="G337" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="H337" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I337" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="338" customHeight="1" spans="1:9">
+      <c r="A338" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C338" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D338" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E338" s="1">
+        <v>170.9</v>
+      </c>
+      <c r="F338" s="1">
+        <v>178.9</v>
+      </c>
+      <c r="G338" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="H338" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I338" s="1">
+        <v>17.9</v>
+      </c>
+    </row>
+    <row r="339" customHeight="1" spans="1:9">
+      <c r="A339" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C339" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D339" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E339" s="1">
+        <v>168.7</v>
+      </c>
+      <c r="F339" s="1">
+        <v>176.3</v>
+      </c>
+      <c r="G339" s="1">
+        <v>4.4</v>
+      </c>
+      <c r="H339" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I339" s="1">
+        <v>16.1</v>
+      </c>
+    </row>
+    <row r="340" customHeight="1" spans="1:9">
+      <c r="A340" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C340" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D340" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E340" s="1">
+        <v>220.4</v>
+      </c>
+      <c r="F340" s="1">
+        <v>227.1</v>
+      </c>
+      <c r="G340" s="1">
+        <v>3</v>
+      </c>
+      <c r="H340" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I340" s="1">
+        <v>49.6</v>
+      </c>
+    </row>
+    <row r="341" customHeight="1" spans="1:9">
+      <c r="A341" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C341" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D341" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E341" s="1">
+        <v>212.6</v>
+      </c>
+      <c r="F341" s="1">
+        <v>217.3</v>
+      </c>
+      <c r="G341" s="1">
+        <v>2.2</v>
+      </c>
+      <c r="H341" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I341" s="1">
+        <v>43.2</v>
+      </c>
+    </row>
+    <row r="342" customHeight="1" spans="1:9">
+      <c r="A342" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B342" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C342" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D342" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E342" s="1">
+        <v>199.9</v>
+      </c>
+      <c r="F342" s="1">
+        <v>198</v>
+      </c>
+      <c r="G342" s="1">
+        <v>-0.9</v>
+      </c>
+      <c r="H342" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I342" s="1">
+        <v>30.4</v>
+      </c>
+    </row>
+    <row r="343" customHeight="1" spans="1:9">
+      <c r="A343" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C343" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D343" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E343" s="1">
+        <v>182.4</v>
+      </c>
+      <c r="F343" s="1">
+        <v>178.9</v>
+      </c>
+      <c r="G343" s="1">
+        <v>-1.9</v>
+      </c>
+      <c r="H343" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I343" s="1">
+        <v>17.8</v>
+      </c>
+    </row>
+    <row r="344" customHeight="1" spans="1:9">
+      <c r="A344" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B344" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C344" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D344" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E344" s="1">
+        <v>226.1</v>
+      </c>
+      <c r="F344" s="1">
+        <v>217</v>
+      </c>
+      <c r="G344" s="1">
+        <v>-4</v>
+      </c>
+      <c r="H344" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I344" s="1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="345" customHeight="1" spans="1:9">
+      <c r="A345" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C345" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D345" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E345" s="1">
+        <v>216.2</v>
+      </c>
+      <c r="F345" s="1">
+        <v>206.1</v>
+      </c>
+      <c r="G345" s="1">
+        <v>-4.6</v>
+      </c>
+      <c r="H345" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I345" s="1">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="346" customHeight="1" spans="1:9">
+      <c r="A346" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C346" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D346" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E346" s="1">
+        <v>200</v>
+      </c>
+      <c r="F346" s="1">
+        <v>187.6</v>
+      </c>
+      <c r="G346" s="1">
+        <v>-6.1</v>
+      </c>
+      <c r="H346" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I346" s="1">
+        <v>23.6</v>
+      </c>
+    </row>
+    <row r="347" customHeight="1" spans="1:9">
+      <c r="A347" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C347" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D347" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E347" s="1">
+        <v>185.4</v>
+      </c>
+      <c r="F347" s="1">
+        <v>173.6</v>
+      </c>
+      <c r="G347" s="1">
+        <v>-6.3</v>
+      </c>
+      <c r="H347" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I347" s="1">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="348" customHeight="1" spans="1:9">
+      <c r="A348" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C348" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D348" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E348" s="1">
+        <v>200.2</v>
+      </c>
+      <c r="F348" s="1">
+        <v>177.3</v>
+      </c>
+      <c r="G348" s="1">
+        <v>-11.4</v>
+      </c>
+      <c r="H348" s="1">
+        <v>151.7</v>
+      </c>
+      <c r="I348" s="1">
+        <v>16.8</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H167" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:H219" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update: 2026/06/29 周一  9:34:48.69
</commit_message>
<xml_diff>
--- a/source/8、绩效异常岗位/1、装车岗/装车岗-6月.xlsx
+++ b/source/8、绩效异常岗位/1、装车岗/装车岗-6月.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I466"/>
+  <dimension ref="A1:I571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18112,6 +18112,3927 @@
         <v>15.5</v>
       </c>
     </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>河南区</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>商丘</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>128.2</v>
+      </c>
+      <c r="F467" t="n">
+        <v>157</v>
+      </c>
+      <c r="G467" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="H467" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I467" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>河北区</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>石家庄</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="F468" t="n">
+        <v>168.8</v>
+      </c>
+      <c r="G468" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="H468" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I468" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>河北区</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>邢邯</t>
+        </is>
+      </c>
+      <c r="E469" t="n">
+        <v>133</v>
+      </c>
+      <c r="F469" t="n">
+        <v>149.3</v>
+      </c>
+      <c r="G469" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>浙北区</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>东方天地港</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>166</v>
+      </c>
+      <c r="F470" t="n">
+        <v>184.1</v>
+      </c>
+      <c r="G470" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H470" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I470" t="n">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>甘肃区</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>兰州</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="F471" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="G471" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>宁夏区</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>银川</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>126.9</v>
+      </c>
+      <c r="F472" t="n">
+        <v>140.2</v>
+      </c>
+      <c r="G472" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>义乌</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>219.3</v>
+      </c>
+      <c r="F473" t="n">
+        <v>239.2</v>
+      </c>
+      <c r="G473" t="n">
+        <v>9</v>
+      </c>
+      <c r="H473" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I473" t="n">
+        <v>57.9</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>淮安</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="F474" t="n">
+        <v>198</v>
+      </c>
+      <c r="G474" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="H474" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I474" t="n">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>南通</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="F475" t="n">
+        <v>176.7</v>
+      </c>
+      <c r="G475" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H475" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I475" t="n">
+        <v>16.6</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>临海</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>168.7</v>
+      </c>
+      <c r="F476" t="n">
+        <v>174</v>
+      </c>
+      <c r="G476" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H476" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I476" t="n">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>贵州区</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>贵阳</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="F477" t="n">
+        <v>219</v>
+      </c>
+      <c r="G477" t="n">
+        <v>3</v>
+      </c>
+      <c r="H477" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I477" t="n">
+        <v>44.6</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>四川区</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>成都</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>220.4</v>
+      </c>
+      <c r="F478" t="n">
+        <v>225.2</v>
+      </c>
+      <c r="G478" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H478" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I478" t="n">
+        <v>48.7</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>重庆区</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="E479" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="F479" t="n">
+        <v>195.1</v>
+      </c>
+      <c r="G479" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="H479" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I479" t="n">
+        <v>28.8</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>合肥</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="F480" t="n">
+        <v>175.4</v>
+      </c>
+      <c r="G480" t="n">
+        <v>-3.8</v>
+      </c>
+      <c r="H480" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I480" t="n">
+        <v>15.8</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>广东区</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>226.1</v>
+      </c>
+      <c r="F481" t="n">
+        <v>216.8</v>
+      </c>
+      <c r="G481" t="n">
+        <v>-4.1</v>
+      </c>
+      <c r="H481" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I481" t="n">
+        <v>43.1</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>粤东区</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>揭阳</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="F482" t="n">
+        <v>206</v>
+      </c>
+      <c r="G482" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="H482" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I482" t="n">
+        <v>35.9</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>南京</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>200</v>
+      </c>
+      <c r="F483" t="n">
+        <v>189.3</v>
+      </c>
+      <c r="G483" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="H483" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I483" t="n">
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>芜湖</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="F484" t="n">
+        <v>173.8</v>
+      </c>
+      <c r="G484" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="H484" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I484" t="n">
+        <v>14.7</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>山东区</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>临沂</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>200.2</v>
+      </c>
+      <c r="F485" t="n">
+        <v>175.1</v>
+      </c>
+      <c r="G485" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="H485" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="I485" t="n">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>河南区</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>商丘</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>128.2</v>
+      </c>
+      <c r="F486" t="n">
+        <v>156.7</v>
+      </c>
+      <c r="G486" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="H486" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I486" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>河北区</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>石家庄</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="F487" t="n">
+        <v>168.8</v>
+      </c>
+      <c r="G487" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H487" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I487" t="n">
+        <v>11.6</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>宁夏区</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>银川</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>126.9</v>
+      </c>
+      <c r="F488" t="n">
+        <v>140.5</v>
+      </c>
+      <c r="G488" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>浙北区</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>东方天地港</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>166</v>
+      </c>
+      <c r="F489" t="n">
+        <v>183.6</v>
+      </c>
+      <c r="G489" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H489" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I489" t="n">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>甘肃区</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>兰州</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="F490" t="n">
+        <v>109.8</v>
+      </c>
+      <c r="G490" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>义乌</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>219.3</v>
+      </c>
+      <c r="F491" t="n">
+        <v>239.3</v>
+      </c>
+      <c r="G491" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H491" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I491" t="n">
+        <v>58.3</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>淮安</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="F492" t="n">
+        <v>197.3</v>
+      </c>
+      <c r="G492" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="H492" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I492" t="n">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>南通</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="F493" t="n">
+        <v>176.7</v>
+      </c>
+      <c r="G493" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H493" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I493" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>贵州区</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>贵阳</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="F494" t="n">
+        <v>219</v>
+      </c>
+      <c r="G494" t="n">
+        <v>3</v>
+      </c>
+      <c r="H494" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I494" t="n">
+        <v>44.9</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>临海</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>168.7</v>
+      </c>
+      <c r="F495" t="n">
+        <v>173.7</v>
+      </c>
+      <c r="G495" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H495" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I495" t="n">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>四川区</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>成都</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>220.4</v>
+      </c>
+      <c r="F496" t="n">
+        <v>224.7</v>
+      </c>
+      <c r="G496" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H496" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I496" t="n">
+        <v>48.6</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>重庆区</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="F497" t="n">
+        <v>194.7</v>
+      </c>
+      <c r="G497" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="H497" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I497" t="n">
+        <v>28.8</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>合肥</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="F498" t="n">
+        <v>174.6</v>
+      </c>
+      <c r="G498" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="H498" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I498" t="n">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>广东区</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="E499" t="n">
+        <v>226.1</v>
+      </c>
+      <c r="F499" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="G499" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="H499" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I499" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>粤东区</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>揭阳</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="F500" t="n">
+        <v>205.9</v>
+      </c>
+      <c r="G500" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="H500" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I500" t="n">
+        <v>36.2</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>南京</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>200</v>
+      </c>
+      <c r="F501" t="n">
+        <v>189.2</v>
+      </c>
+      <c r="G501" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="H501" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I501" t="n">
+        <v>25.2</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>芜湖</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="F502" t="n">
+        <v>173.6</v>
+      </c>
+      <c r="G502" t="n">
+        <v>-6.3</v>
+      </c>
+      <c r="H502" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I502" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>山东区</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>临沂</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>200.2</v>
+      </c>
+      <c r="F503" t="n">
+        <v>174.7</v>
+      </c>
+      <c r="G503" t="n">
+        <v>-12.7</v>
+      </c>
+      <c r="H503" t="n">
+        <v>151.1</v>
+      </c>
+      <c r="I503" t="n">
+        <v>15.5</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>河南区</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>商丘</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>128.2</v>
+      </c>
+      <c r="F504" t="n">
+        <v>156.7</v>
+      </c>
+      <c r="G504" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="H504" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I504" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>河北区</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>石家庄</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="F505" t="n">
+        <v>168.6</v>
+      </c>
+      <c r="G505" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="H505" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I505" t="n">
+        <v>11.7</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>浙北区</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>东方天地港</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>166</v>
+      </c>
+      <c r="F506" t="n">
+        <v>183</v>
+      </c>
+      <c r="G506" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="H506" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I506" t="n">
+        <v>21.3</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>甘肃区</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>兰州</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="F507" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="G507" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>义乌</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>219.3</v>
+      </c>
+      <c r="F508" t="n">
+        <v>241.6</v>
+      </c>
+      <c r="G508" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H508" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I508" t="n">
+        <v>60.1</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>淮安</t>
+        </is>
+      </c>
+      <c r="E509" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="F509" t="n">
+        <v>196.7</v>
+      </c>
+      <c r="G509" t="n">
+        <v>5</v>
+      </c>
+      <c r="H509" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I509" t="n">
+        <v>30.3</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>南通</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="F510" t="n">
+        <v>176.5</v>
+      </c>
+      <c r="G510" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H510" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I510" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>贵州区</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>贵阳</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="F511" t="n">
+        <v>218.6</v>
+      </c>
+      <c r="G511" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H511" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I511" t="n">
+        <v>44.9</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>临海</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>168.7</v>
+      </c>
+      <c r="F512" t="n">
+        <v>173.4</v>
+      </c>
+      <c r="G512" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H512" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I512" t="n">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>四川区</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>成都</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>220.4</v>
+      </c>
+      <c r="F513" t="n">
+        <v>224.4</v>
+      </c>
+      <c r="G513" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H513" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I513" t="n">
+        <v>48.7</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>重庆区</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="F514" t="n">
+        <v>194.5</v>
+      </c>
+      <c r="G514" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="H514" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I514" t="n">
+        <v>28.9</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>广东区</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>226.1</v>
+      </c>
+      <c r="F515" t="n">
+        <v>215.6</v>
+      </c>
+      <c r="G515" t="n">
+        <v>-4.6</v>
+      </c>
+      <c r="H515" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I515" t="n">
+        <v>42.9</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>合肥</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="F516" t="n">
+        <v>173.8</v>
+      </c>
+      <c r="G516" t="n">
+        <v>-4.7</v>
+      </c>
+      <c r="H516" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I516" t="n">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>粤东区</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>揭阳</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="F517" t="n">
+        <v>205.6</v>
+      </c>
+      <c r="G517" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="H517" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I517" t="n">
+        <v>36.3</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>南京</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>200</v>
+      </c>
+      <c r="F518" t="n">
+        <v>188.6</v>
+      </c>
+      <c r="G518" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="H518" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I518" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>芜湖</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="F519" t="n">
+        <v>173.5</v>
+      </c>
+      <c r="G519" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="H519" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I519" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>山东区</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>临沂</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>200.2</v>
+      </c>
+      <c r="F520" t="n">
+        <v>174.2</v>
+      </c>
+      <c r="G520" t="n">
+        <v>-13</v>
+      </c>
+      <c r="H520" t="n">
+        <v>150.8</v>
+      </c>
+      <c r="I520" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>河南区</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>商丘</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>128.2</v>
+      </c>
+      <c r="F521" t="n">
+        <v>156.1</v>
+      </c>
+      <c r="G521" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="H521" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I521" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>河北区</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>石家庄</t>
+        </is>
+      </c>
+      <c r="E522" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="F522" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="G522" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="H522" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I522" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>义乌</t>
+        </is>
+      </c>
+      <c r="E523" t="n">
+        <v>219</v>
+      </c>
+      <c r="F523" t="n">
+        <v>242.9</v>
+      </c>
+      <c r="G523" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="H523" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I523" t="n">
+        <v>61.3</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>甘肃区</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>兰州</t>
+        </is>
+      </c>
+      <c r="E524" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="F524" t="n">
+        <v>109.6</v>
+      </c>
+      <c r="G524" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>浙北区</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>东方天地港</t>
+        </is>
+      </c>
+      <c r="E525" t="n">
+        <v>166</v>
+      </c>
+      <c r="F525" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="G525" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H525" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I525" t="n">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>淮安</t>
+        </is>
+      </c>
+      <c r="E526" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="F526" t="n">
+        <v>195.7</v>
+      </c>
+      <c r="G526" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H526" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I526" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>南通</t>
+        </is>
+      </c>
+      <c r="E527" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="F527" t="n">
+        <v>176.6</v>
+      </c>
+      <c r="G527" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H527" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I527" t="n">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>临海</t>
+        </is>
+      </c>
+      <c r="E528" t="n">
+        <v>168.7</v>
+      </c>
+      <c r="F528" t="n">
+        <v>173.3</v>
+      </c>
+      <c r="G528" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H528" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I528" t="n">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>贵州区</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>贵阳</t>
+        </is>
+      </c>
+      <c r="E529" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="F529" t="n">
+        <v>217.9</v>
+      </c>
+      <c r="G529" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H529" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I529" t="n">
+        <v>44.7</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>四川区</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>成都</t>
+        </is>
+      </c>
+      <c r="E530" t="n">
+        <v>220.4</v>
+      </c>
+      <c r="F530" t="n">
+        <v>224.3</v>
+      </c>
+      <c r="G530" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H530" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I530" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>重庆区</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="E531" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="F531" t="n">
+        <v>194.5</v>
+      </c>
+      <c r="G531" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="H531" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I531" t="n">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>广东区</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>226.1</v>
+      </c>
+      <c r="F532" t="n">
+        <v>215</v>
+      </c>
+      <c r="G532" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="H532" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I532" t="n">
+        <v>42.8</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>粤东区</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>揭阳</t>
+        </is>
+      </c>
+      <c r="E533" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="F533" t="n">
+        <v>205.5</v>
+      </c>
+      <c r="G533" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="H533" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I533" t="n">
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>合肥</t>
+        </is>
+      </c>
+      <c r="E534" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="F534" t="n">
+        <v>172.9</v>
+      </c>
+      <c r="G534" t="n">
+        <v>-5.1</v>
+      </c>
+      <c r="H534" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I534" t="n">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>南京</t>
+        </is>
+      </c>
+      <c r="E535" t="n">
+        <v>200</v>
+      </c>
+      <c r="F535" t="n">
+        <v>187.9</v>
+      </c>
+      <c r="G535" t="n">
+        <v>-6</v>
+      </c>
+      <c r="H535" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I535" t="n">
+        <v>24.8</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>芜湖</t>
+        </is>
+      </c>
+      <c r="E536" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="F536" t="n">
+        <v>173.2</v>
+      </c>
+      <c r="G536" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="H536" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I536" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>山东区</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>临沂</t>
+        </is>
+      </c>
+      <c r="E537" t="n">
+        <v>200.2</v>
+      </c>
+      <c r="F537" t="n">
+        <v>173.8</v>
+      </c>
+      <c r="G537" t="n">
+        <v>-13.1</v>
+      </c>
+      <c r="H537" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="I537" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>河南区</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>商丘</t>
+        </is>
+      </c>
+      <c r="E538" t="n">
+        <v>128.2</v>
+      </c>
+      <c r="F538" t="n">
+        <v>155.9</v>
+      </c>
+      <c r="G538" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="H538" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I538" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>河北区</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>石家庄</t>
+        </is>
+      </c>
+      <c r="E539" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="F539" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="G539" t="n">
+        <v>13</v>
+      </c>
+      <c r="H539" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I539" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>义乌</t>
+        </is>
+      </c>
+      <c r="E540" t="n">
+        <v>219</v>
+      </c>
+      <c r="F540" t="n">
+        <v>242.2</v>
+      </c>
+      <c r="G540" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H540" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I540" t="n">
+        <v>61.2</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>甘肃区</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>兰州</t>
+        </is>
+      </c>
+      <c r="E541" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="F541" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="G541" t="n">
+        <v>10</v>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>浙北区</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>东方天地港</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>166</v>
+      </c>
+      <c r="F542" t="n">
+        <v>182.1</v>
+      </c>
+      <c r="G542" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H542" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I542" t="n">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>淮安</t>
+        </is>
+      </c>
+      <c r="E543" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="F543" t="n">
+        <v>195.1</v>
+      </c>
+      <c r="G543" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H543" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I543" t="n">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>南通</t>
+        </is>
+      </c>
+      <c r="E544" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="F544" t="n">
+        <v>176.4</v>
+      </c>
+      <c r="G544" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H544" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I544" t="n">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>临海</t>
+        </is>
+      </c>
+      <c r="E545" t="n">
+        <v>168.7</v>
+      </c>
+      <c r="F545" t="n">
+        <v>173</v>
+      </c>
+      <c r="G545" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H545" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I545" t="n">
+        <v>15.2</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>贵州区</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>贵阳</t>
+        </is>
+      </c>
+      <c r="E546" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="F546" t="n">
+        <v>217.3</v>
+      </c>
+      <c r="G546" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H546" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I546" t="n">
+        <v>44.7</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>四川区</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>成都</t>
+        </is>
+      </c>
+      <c r="E547" t="n">
+        <v>220.4</v>
+      </c>
+      <c r="F547" t="n">
+        <v>224.1</v>
+      </c>
+      <c r="G547" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H547" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I547" t="n">
+        <v>49.2</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>重庆区</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="E548" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="F548" t="n">
+        <v>194.4</v>
+      </c>
+      <c r="G548" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="H548" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I548" t="n">
+        <v>29.4</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>粤东区</t>
+        </is>
+      </c>
+      <c r="D549" t="inlineStr">
+        <is>
+          <t>揭阳</t>
+        </is>
+      </c>
+      <c r="E549" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="F549" t="n">
+        <v>205.1</v>
+      </c>
+      <c r="G549" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H549" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I549" t="n">
+        <v>36.6</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>广东区</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="E550" t="n">
+        <v>226.1</v>
+      </c>
+      <c r="F550" t="n">
+        <v>214.3</v>
+      </c>
+      <c r="G550" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="H550" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I550" t="n">
+        <v>42.7</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>合肥</t>
+        </is>
+      </c>
+      <c r="E551" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="F551" t="n">
+        <v>172.7</v>
+      </c>
+      <c r="G551" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="H551" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I551" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>南京</t>
+        </is>
+      </c>
+      <c r="E552" t="n">
+        <v>200</v>
+      </c>
+      <c r="F552" t="n">
+        <v>187.7</v>
+      </c>
+      <c r="G552" t="n">
+        <v>-6.1</v>
+      </c>
+      <c r="H552" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I552" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>芜湖</t>
+        </is>
+      </c>
+      <c r="E553" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="F553" t="n">
+        <v>172.8</v>
+      </c>
+      <c r="G553" t="n">
+        <v>-6.8</v>
+      </c>
+      <c r="H553" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I553" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>山东区</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>临沂</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>200.2</v>
+      </c>
+      <c r="F554" t="n">
+        <v>173.3</v>
+      </c>
+      <c r="G554" t="n">
+        <v>-13.4</v>
+      </c>
+      <c r="H554" t="n">
+        <v>150.1</v>
+      </c>
+      <c r="I554" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>河南区</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>商丘</t>
+        </is>
+      </c>
+      <c r="E555" t="n">
+        <v>129.4</v>
+      </c>
+      <c r="F555" t="n">
+        <v>155.4</v>
+      </c>
+      <c r="G555" t="n">
+        <v>20</v>
+      </c>
+      <c r="H555" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I555" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>河北区</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>石家庄</t>
+        </is>
+      </c>
+      <c r="E556" t="n">
+        <v>148.5</v>
+      </c>
+      <c r="F556" t="n">
+        <v>167.5</v>
+      </c>
+      <c r="G556" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="H556" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I556" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>义乌</t>
+        </is>
+      </c>
+      <c r="E557" t="n">
+        <v>219</v>
+      </c>
+      <c r="F557" t="n">
+        <v>241.3</v>
+      </c>
+      <c r="G557" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H557" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I557" t="n">
+        <v>61.1</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>甘肃区</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>兰州</t>
+        </is>
+      </c>
+      <c r="E558" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="F558" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="G558" t="n">
+        <v>10</v>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>浙北区</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>东方天地港</t>
+        </is>
+      </c>
+      <c r="E559" t="n">
+        <v>166</v>
+      </c>
+      <c r="F559" t="n">
+        <v>181.9</v>
+      </c>
+      <c r="G559" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H559" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I559" t="n">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>浙南区</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>临海</t>
+        </is>
+      </c>
+      <c r="E560" t="n">
+        <v>165.9</v>
+      </c>
+      <c r="F560" t="n">
+        <v>172.9</v>
+      </c>
+      <c r="G560" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H560" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I560" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>淮安</t>
+        </is>
+      </c>
+      <c r="E561" t="n">
+        <v>187.3</v>
+      </c>
+      <c r="F561" t="n">
+        <v>194.6</v>
+      </c>
+      <c r="G561" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="H561" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I561" t="n">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>南通</t>
+        </is>
+      </c>
+      <c r="E562" t="n">
+        <v>170.9</v>
+      </c>
+      <c r="F562" t="n">
+        <v>175.9</v>
+      </c>
+      <c r="G562" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H562" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I562" t="n">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>贵州区</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>贵阳</t>
+        </is>
+      </c>
+      <c r="E563" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="F563" t="n">
+        <v>216.9</v>
+      </c>
+      <c r="G563" t="n">
+        <v>2</v>
+      </c>
+      <c r="H563" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I563" t="n">
+        <v>44.8</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>四川区</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>成都</t>
+        </is>
+      </c>
+      <c r="E564" t="n">
+        <v>220.4</v>
+      </c>
+      <c r="F564" t="n">
+        <v>223.5</v>
+      </c>
+      <c r="G564" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H564" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I564" t="n">
+        <v>49.2</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>重庆区</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="E565" t="n">
+        <v>199.9</v>
+      </c>
+      <c r="F565" t="n">
+        <v>194.1</v>
+      </c>
+      <c r="G565" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="H565" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I565" t="n">
+        <v>29.6</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>粤东区</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>揭阳</t>
+        </is>
+      </c>
+      <c r="E566" t="n">
+        <v>216.2</v>
+      </c>
+      <c r="F566" t="n">
+        <v>204.7</v>
+      </c>
+      <c r="G566" t="n">
+        <v>-5.2</v>
+      </c>
+      <c r="H566" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I566" t="n">
+        <v>36.7</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>合肥</t>
+        </is>
+      </c>
+      <c r="E567" t="n">
+        <v>182.4</v>
+      </c>
+      <c r="F567" t="n">
+        <v>172.1</v>
+      </c>
+      <c r="G567" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="H567" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I567" t="n">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>广东区</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="E568" t="n">
+        <v>226.1</v>
+      </c>
+      <c r="F568" t="n">
+        <v>213.5</v>
+      </c>
+      <c r="G568" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="H568" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I568" t="n">
+        <v>42.5</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>江苏区</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>南京</t>
+        </is>
+      </c>
+      <c r="E569" t="n">
+        <v>200</v>
+      </c>
+      <c r="F569" t="n">
+        <v>187.5</v>
+      </c>
+      <c r="G569" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="H569" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I569" t="n">
+        <v>25.2</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>安徽区</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>芜湖</t>
+        </is>
+      </c>
+      <c r="E570" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="F570" t="n">
+        <v>171.9</v>
+      </c>
+      <c r="G570" t="n">
+        <v>-7.2</v>
+      </c>
+      <c r="H570" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I570" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>装车岗</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>山东区</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>临沂</t>
+        </is>
+      </c>
+      <c r="E571" t="n">
+        <v>200.2</v>
+      </c>
+      <c r="F571" t="n">
+        <v>172.8</v>
+      </c>
+      <c r="G571" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="H571" t="n">
+        <v>149.7</v>
+      </c>
+      <c r="I571" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>